<commit_message>
docs: synchronize runbook with official SIST CSE AI Capstone specifications and rubric
</commit_message>
<xml_diff>
--- a/docs/Student_FullStack_Project_Runbook.xlsx
+++ b/docs/Student_FullStack_Project_Runbook.xlsx
@@ -28,7 +28,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="6">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -52,7 +52,7 @@
       <name val="Calibri"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
-      <sz val="11"/>
+      <sz val="12"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -65,8 +65,20 @@
       <color rgb="000F172A"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="001E3A8A"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -91,8 +103,14 @@
         <bgColor rgb="00334155"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E0E7FF"/>
+        <bgColor rgb="00E0E7FF"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -114,21 +132,58 @@
         <color rgb="00CBD5E1"/>
       </bottom>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00CBD5E1"/>
+      </left>
+      <right style="thin">
+        <color rgb="00CBD5E1"/>
+      </right>
+      <top style="thin">
+        <color rgb="00CBD5E1"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="001E3A8A"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -507,161 +562,445 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B14"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:D29"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
-    <col width="48" customWidth="1" min="1" max="1"/>
-    <col width="48" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="44" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="24" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>SMART STATIONERY INVENTORY MANAGEMENT SYSTEM</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
+          <t>🎓 SATHYABAMA INSTITUTE OF SCIENCE AND TECHNOLOGY (SIST)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Full-Stack College Project Academic Runbook (SOP-COLLEGE-FSD-2026)</t>
-        </is>
-      </c>
-    </row>
-    <row r="3"/>
-    <row r="4">
+          <t>Department of Computer Science and Engineering — Artificial Intelligence (CSE AI) | Capstone Runbook</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="26" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Field</t>
-        </is>
-      </c>
-      <c r="B4" s="3" t="inlineStr">
-        <is>
-          <t>Project Specification Details</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
+          <t>📌 CAPSTONE PROJECT CHARTER &amp; TEAM SPECIFICATIONS</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="22" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>Project Title</t>
+          <t>Student 1 (Lead / Full Name):</t>
         </is>
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
+          <t>Nikhila V</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>Student 1 Register No:</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>44731059</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="22" customHeight="1">
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>Student 2 (Partner Full Name):</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>Zaid Basha</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="inlineStr">
+        <is>
+          <t>Student 2 Register No:</t>
+        </is>
+      </c>
+      <c r="D6" s="7" t="inlineStr">
+        <is>
+          <t>44731049</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="22" customHeight="1">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Department &amp; Year:</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>B.E. CSE (Artificial Intelligence) — 3rd Year</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>Batch / Section:</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>2023 - 2027 / Section A4</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="22" customHeight="1">
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>Official Project Title:</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="inlineStr">
+        <is>
           <t>Smart Stationery Inventory Management System</t>
         </is>
       </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="6" t="inlineStr">
-        <is>
-          <t>Team ID</t>
-        </is>
-      </c>
-      <c r="B6" s="7" t="inlineStr">
-        <is>
-          <t>TEAM-FSD-04</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>Department</t>
-        </is>
-      </c>
-      <c r="B7" s="5" t="inlineStr">
-        <is>
-          <t>Computer Science and Engineering</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="6" t="inlineStr">
-        <is>
-          <t>Academic Year</t>
-        </is>
-      </c>
-      <c r="B8" s="7" t="inlineStr">
-        <is>
-          <t>2025 - 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
+      <c r="C8" s="6" t="inlineStr">
+        <is>
+          <t>Project Domain:</t>
+        </is>
+      </c>
+      <c r="D8" s="7" t="inlineStr">
+        <is>
+          <t>Full-Stack Web + AI Application</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="22" customHeight="1">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>Date of Submission</t>
+          <t>Primary Technology Stack:</t>
         </is>
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
+          <t>Core Java 21, JDBC, MySQL 8.0, React 19, RESTful API, HTML5, CSS3, Vite</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>Project Trainer / Mentor:</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>Placement Training Cell / Trainer</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="22" customHeight="1">
       <c r="A10" s="6" t="inlineStr">
         <is>
-          <t>Student 1 (Lead Architect)</t>
+          <t>Sprint Start Date:</t>
         </is>
       </c>
       <c r="B10" s="7" t="inlineStr">
         <is>
-          <t>Nikhila V (Register Number: 44731059)</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
+          <t>2026-09-18 (Phase 1: Define Kickoff)</t>
+        </is>
+      </c>
+      <c r="C10" s="6" t="inlineStr">
+        <is>
+          <t>Target Deployment &amp; Viva Date:</t>
+        </is>
+      </c>
+      <c r="D10" s="7" t="inlineStr">
+        <is>
+          <t>Phase 4: Final Viva &amp; Cloud Pitch</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="22" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>Student 2 (Backend &amp; DB Specialist)</t>
+          <t>Active GitHub Repository:</t>
         </is>
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>Zaid Basha (Register Number: 44731049)</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="6" t="inlineStr">
-        <is>
-          <t>Project Architecture</t>
-        </is>
-      </c>
-      <c r="B12" s="7" t="inlineStr">
-        <is>
-          <t>3-Tier (Vanilla HTML5/CSS3/JS -&gt; Java 21 SE -&gt; MySQL 8.0)</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="4" t="inlineStr">
-        <is>
-          <t>Approved Tech Stack</t>
-        </is>
-      </c>
-      <c r="B13" s="5" t="inlineStr">
-        <is>
-          <t>HTML5, CSS3, Vanilla JS (ES6+), Core Java 21 (HttpServer / JDBC), MySQL 8.0</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="6" t="inlineStr">
-        <is>
-          <t>Prohibited Frameworks</t>
-        </is>
-      </c>
-      <c r="B14" s="7" t="inlineStr">
-        <is>
-          <t>No Spring Boot, No React, No Angular, No Node.js, No Tailwind, No MongoDB</t>
-        </is>
+          <t>https://github.com/Nikki060927/Inventory-Management-System</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>Live Deployment URLs:</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>http://127.0.0.1:5173 (React) &amp; :8080 (API)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="26" customHeight="1">
+      <c r="A13" s="8" t="inlineStr">
+        <is>
+          <t>📖 RUNBOOK INSTRUCTIONS &amp; CARE PROMPTING GUIDELINES</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="21" customHeight="1">
+      <c r="A14" s="9" t="inlineStr">
+        <is>
+          <t>1.</t>
+        </is>
+      </c>
+      <c r="B14" s="10" t="inlineStr">
+        <is>
+          <t>This Runbook is your official engineering portfolio record for Sathyabama Institute of Science and Technology (SIST).</t>
+        </is>
+      </c>
+      <c r="C14" s="11" t="n"/>
+      <c r="D14" s="11" t="n"/>
+    </row>
+    <row r="15" ht="21" customHeight="1">
+      <c r="A15" s="12" t="inlineStr">
+        <is>
+          <t>2.</t>
+        </is>
+      </c>
+      <c r="B15" s="13" t="inlineStr">
+        <is>
+          <t>Execute across the 4 Disciplined SDLC Phases: Phase 1 (Define) -&gt; Phase 2 (Design) -&gt; Phase 3 (Develop) -&gt; Phase 4 (Deploy).</t>
+        </is>
+      </c>
+      <c r="C15" s="14" t="n"/>
+      <c r="D15" s="14" t="n"/>
+    </row>
+    <row r="16" ht="21" customHeight="1">
+      <c r="A16" s="9" t="inlineStr">
+        <is>
+          <t>3.</t>
+        </is>
+      </c>
+      <c r="B16" s="10" t="inlineStr">
+        <is>
+          <t>Apply the CARE Formula for all AI prompts: C (Context) -&gt; A (Action) -&gt; R (Result) -&gt; E (Example/Clarification).</t>
+        </is>
+      </c>
+      <c r="C16" s="11" t="n"/>
+      <c r="D16" s="11" t="n"/>
+    </row>
+    <row r="17" ht="21" customHeight="1">
+      <c r="A17" s="12" t="inlineStr">
+        <is>
+          <t>4.</t>
+        </is>
+      </c>
+      <c r="B17" s="13" t="inlineStr">
+        <is>
+          <t>In Phase 2, model 3-tier System Architecture and 3NF Relational Database Schemas on Draw.io (https://app.diagrams.net).</t>
+        </is>
+      </c>
+      <c r="C17" s="14" t="n"/>
+      <c r="D17" s="14" t="n"/>
+    </row>
+    <row r="18" ht="21" customHeight="1">
+      <c r="A18" s="9" t="inlineStr">
+        <is>
+          <t>5.</t>
+        </is>
+      </c>
+      <c r="B18" s="10" t="inlineStr">
+        <is>
+          <t>In Phase 3, build robust Spring Boot 3 / Core Java REST APIs, MySQL JPA/JDBC persistence, and responsive HTML5/CSS Grid / React frontends.</t>
+        </is>
+      </c>
+      <c r="C18" s="11" t="n"/>
+      <c r="D18" s="11" t="n"/>
+    </row>
+    <row r="19" ht="21" customHeight="1">
+      <c r="A19" s="12" t="inlineStr">
+        <is>
+          <t>6.</t>
+        </is>
+      </c>
+      <c r="B19" s="13" t="inlineStr">
+        <is>
+          <t>In Phase 4, resolve all CORS &amp; HTTP issues, package a 1-click startup script, and deliver a live 3-minute technical viva pitch.</t>
+        </is>
+      </c>
+      <c r="C19" s="14" t="n"/>
+      <c r="D19" s="14" t="n"/>
+    </row>
+    <row r="20" ht="21" customHeight="1">
+      <c r="A20" s="9" t="inlineStr">
+        <is>
+          <t>7.</t>
+        </is>
+      </c>
+      <c r="B20" s="10" t="inlineStr">
+        <is>
+          <t>Replace all placeholder brackets '[FILL HERE]' with your team's actual code, diagrams, API JSON, and active GitHub URLs.</t>
+        </is>
+      </c>
+      <c r="C20" s="11" t="n"/>
+      <c r="D20" s="11" t="n"/>
+    </row>
+    <row r="22" ht="26" customHeight="1">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>📊 SIST CSE AI EVALUATION &amp; VIVA RUBRIC (100 MARKS TOTAL)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="26" customHeight="1">
+      <c r="A23" s="15" t="inlineStr">
+        <is>
+          <t>SDLC Phase</t>
+        </is>
+      </c>
+      <c r="B23" s="15" t="inlineStr">
+        <is>
+          <t>Evaluation Criteria &amp; Milestone Deliverable</t>
+        </is>
+      </c>
+      <c r="C23" s="15" t="inlineStr">
+        <is>
+          <t>Max Marks</t>
+        </is>
+      </c>
+      <c r="D23" s="15" t="inlineStr">
+        <is>
+          <t>Evaluator Score</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="22" customHeight="1">
+      <c r="A24" s="6" t="inlineStr">
+        <is>
+          <t>Phase 1: DEFINE</t>
+        </is>
+      </c>
+      <c r="B24" s="7" t="inlineStr">
+        <is>
+          <t>Problem statement, user personas, Given/When/Then acceptance criteria</t>
+        </is>
+      </c>
+      <c r="C24" s="9" t="n">
+        <v>15</v>
+      </c>
+      <c r="D24" s="9" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="25" ht="22" customHeight="1">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>Phase 2: DESIGN</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="inlineStr">
+        <is>
+          <t>Draw.io system architecture diagram, 3NF MySQL schema, REST API contracts</t>
+        </is>
+      </c>
+      <c r="C25" s="12" t="n">
+        <v>20</v>
+      </c>
+      <c r="D25" s="12" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="26" ht="22" customHeight="1">
+      <c r="A26" s="6" t="inlineStr">
+        <is>
+          <t>Phase 3: DEVELOP</t>
+        </is>
+      </c>
+      <c r="B26" s="7" t="inlineStr">
+        <is>
+          <t>Responsive Frontend UI (HTML5, CSS Grid / React), REST API &amp; JDBC/JPA</t>
+        </is>
+      </c>
+      <c r="C26" s="9" t="n">
+        <v>25</v>
+      </c>
+      <c r="D26" s="9" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="27" ht="22" customHeight="1">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>Phase 3: INTEGRATE</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="inlineStr">
+        <is>
+          <t>MySQL database persistence, JavaScript Fetch API &amp; CORS resolution</t>
+        </is>
+      </c>
+      <c r="C27" s="12" t="n">
+        <v>20</v>
+      </c>
+      <c r="D27" s="12" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="28" ht="22" customHeight="1">
+      <c r="A28" s="6" t="inlineStr">
+        <is>
+          <t>Phase 4: DEPLOY</t>
+        </is>
+      </c>
+      <c r="B28" s="7" t="inlineStr">
+        <is>
+          <t>Cloud deployment / 1-click startup script, GitHub documentation, 3-min viva pitch</t>
+        </is>
+      </c>
+      <c r="C28" s="9" t="n">
+        <v>20</v>
+      </c>
+      <c r="D28" s="9" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="29" ht="25" customHeight="1">
+      <c r="A29" s="16" t="inlineStr">
+        <is>
+          <t>TOTAL SCORE</t>
+        </is>
+      </c>
+      <c r="B29" s="16" t="inlineStr">
+        <is>
+          <t>Grand Aggregate Score across all Full-Stack Engineering Dimensions</t>
+        </is>
+      </c>
+      <c r="C29" s="17" t="n">
+        <v>100</v>
+      </c>
+      <c r="D29" s="17" t="n">
+        <v>100</v>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="10">
+    <mergeCell ref="B19:D19"/>
+    <mergeCell ref="B14:D14"/>
+    <mergeCell ref="A22:D22"/>
+    <mergeCell ref="A4:D4"/>
+    <mergeCell ref="B17:D17"/>
+    <mergeCell ref="B18:D18"/>
+    <mergeCell ref="A13:D13"/>
+    <mergeCell ref="B15:D15"/>
+    <mergeCell ref="B16:D16"/>
+    <mergeCell ref="B20:D20"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -673,14 +1012,14 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:F8"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
-    <col width="48" customWidth="1" min="1" max="1"/>
-    <col width="39" customWidth="1" min="2" max="2"/>
+    <col width="49" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
     <col width="43" customWidth="1" min="3" max="3"/>
-    <col width="48" customWidth="1" min="4" max="4"/>
-    <col width="48" customWidth="1" min="5" max="5"/>
-    <col width="48" customWidth="1" min="6" max="6"/>
+    <col width="55" customWidth="1" min="4" max="4"/>
+    <col width="55" customWidth="1" min="5" max="5"/>
+    <col width="55" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -691,195 +1030,195 @@
       </c>
     </row>
     <row r="2"/>
-    <row r="3" ht="25" customHeight="1">
-      <c r="A3" s="8" t="inlineStr">
+    <row r="3" ht="26" customHeight="1">
+      <c r="A3" s="15" t="inlineStr">
         <is>
           <t>Integration Flow</t>
         </is>
       </c>
-      <c r="B3" s="8" t="inlineStr">
-        <is>
-          <t>Frontend Trigger (script.js)</t>
-        </is>
-      </c>
-      <c r="C3" s="8" t="inlineStr">
+      <c r="B3" s="15" t="inlineStr">
+        <is>
+          <t>Frontend Trigger</t>
+        </is>
+      </c>
+      <c r="C3" s="15" t="inlineStr">
         <is>
           <t>HTTP Request Details</t>
         </is>
       </c>
-      <c r="D3" s="8" t="inlineStr">
+      <c r="D3" s="15" t="inlineStr">
         <is>
           <t>Backend Processing (Java)</t>
         </is>
       </c>
-      <c r="E3" s="8" t="inlineStr">
+      <c r="E3" s="15" t="inlineStr">
         <is>
           <t>Database Execution</t>
         </is>
       </c>
-      <c r="F3" s="8" t="inlineStr">
-        <is>
-          <t>DOM Update Mechanism</t>
+      <c r="F3" s="15" t="inlineStr">
+        <is>
+          <t>UI / State Update Mechanism</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="9" t="inlineStr">
+      <c r="A4" s="18" t="inlineStr">
         <is>
           <t>Dashboard KPIs</t>
         </is>
       </c>
-      <c r="B4" s="9" t="inlineStr">
-        <is>
-          <t>DOMContentLoaded -&gt; loadDashboard()</t>
-        </is>
-      </c>
-      <c r="C4" s="9" t="inlineStr">
+      <c r="B4" s="18" t="inlineStr">
+        <is>
+          <t>useEffect() -&gt; fetchKPIs()</t>
+        </is>
+      </c>
+      <c r="C4" s="18" t="inlineStr">
         <is>
           <t>GET /api/reports/dashboard</t>
         </is>
       </c>
-      <c r="D4" s="9" t="inlineStr">
+      <c r="D4" s="18" t="inlineStr">
         <is>
           <t>ReportService aggregates metrics from ProductDAO &amp; SaleDAO</t>
         </is>
       </c>
-      <c r="E4" s="9" t="inlineStr">
+      <c r="E4" s="18" t="inlineStr">
         <is>
           <t>COUNT(), SUM(qty*price) queries in MySQL</t>
         </is>
       </c>
-      <c r="F4" s="9" t="inlineStr">
-        <is>
-          <t>Sets textContent of kpiTotalProducts, kpiValuation, etc.</t>
+      <c r="F4" s="18" t="inlineStr">
+        <is>
+          <t>Updates React kpiData state; renders 4 dynamic metric cards.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="10" t="inlineStr">
+      <c r="A5" s="19" t="inlineStr">
         <is>
           <t>Product Filter</t>
         </is>
       </c>
-      <c r="B5" s="10" t="inlineStr">
-        <is>
-          <t>oninput -&gt; debounceFilterProducts()</t>
-        </is>
-      </c>
-      <c r="C5" s="10" t="inlineStr">
+      <c r="B5" s="19" t="inlineStr">
+        <is>
+          <t>onChange -&gt; debounce search</t>
+        </is>
+      </c>
+      <c r="C5" s="19" t="inlineStr">
         <is>
           <t>GET /api/products?search=...&amp;status=...</t>
         </is>
       </c>
-      <c r="D5" s="10" t="inlineStr">
+      <c r="D5" s="19" t="inlineStr">
         <is>
           <t>SimpleHttpServer parses query string; ProductService filters</t>
         </is>
       </c>
-      <c r="E5" s="10" t="inlineStr">
+      <c r="E5" s="19" t="inlineStr">
         <is>
           <t>SELECT ... WHERE product_name LIKE ? AND status = ?</t>
         </is>
       </c>
-      <c r="F5" s="10" t="inlineStr">
-        <is>
-          <t>Clears and repopulates productsTableBody with status badges.</t>
+      <c r="F5" s="19" t="inlineStr">
+        <is>
+          <t>Updates products array state; rerenders table with color badges.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="9" t="inlineStr">
+      <c r="A6" s="18" t="inlineStr">
         <is>
           <t>Add Product</t>
         </is>
       </c>
-      <c r="B6" s="9" t="inlineStr">
-        <is>
-          <t>onsubmit -&gt; saveProduct(event)</t>
-        </is>
-      </c>
-      <c r="C6" s="9" t="inlineStr">
+      <c r="B6" s="18" t="inlineStr">
+        <is>
+          <t>onSubmit -&gt; handleAddProduct()</t>
+        </is>
+      </c>
+      <c r="C6" s="18" t="inlineStr">
         <is>
           <t>POST /api/products (JSON body)</t>
         </is>
       </c>
-      <c r="D6" s="9" t="inlineStr">
+      <c r="D6" s="18" t="inlineStr">
         <is>
           <t>JsonUtil parses JSON; ProductService validates SKU uniqueness</t>
         </is>
       </c>
-      <c r="E6" s="9" t="inlineStr">
+      <c r="E6" s="18" t="inlineStr">
         <is>
           <t>INSERT INTO products (...) VALUES (?, ?, ...)</t>
         </is>
       </c>
-      <c r="F6" s="9" t="inlineStr">
-        <is>
-          <t>Displays success toast, closes modal, and refreshes catalog table.</t>
+      <c r="F6" s="18" t="inlineStr">
+        <is>
+          <t>Displays success notification, closes modal, and refreshes catalog.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="10" t="inlineStr">
+      <c r="A7" s="19" t="inlineStr">
         <is>
           <t>Inward Stock</t>
         </is>
       </c>
-      <c r="B7" s="10" t="inlineStr">
-        <is>
-          <t>onsubmit -&gt; saveStockAdjustment()</t>
-        </is>
-      </c>
-      <c r="C7" s="10" t="inlineStr">
+      <c r="B7" s="19" t="inlineStr">
+        <is>
+          <t>onSubmit -&gt; recordStock()</t>
+        </is>
+      </c>
+      <c r="C7" s="19" t="inlineStr">
         <is>
           <t>POST /api/stock/inward</t>
         </is>
       </c>
-      <c r="D7" s="10" t="inlineStr">
+      <c r="D7" s="19" t="inlineStr">
         <is>
           <t>StockService updates stock and logs audit record</t>
         </is>
       </c>
-      <c r="E7" s="10" t="inlineStr">
+      <c r="E7" s="19" t="inlineStr">
         <is>
           <t>UPDATE products ...; INSERT INTO stock_transactions ...</t>
         </is>
       </c>
-      <c r="F7" s="10" t="inlineStr">
+      <c r="F7" s="19" t="inlineStr">
         <is>
           <t>Status badge transitions from LOW STOCK (Amber) to IN STOCK (Green).</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="9" t="inlineStr">
+      <c r="A8" s="18" t="inlineStr">
         <is>
           <t>POS Checkout</t>
         </is>
       </c>
-      <c r="B8" s="9" t="inlineStr">
-        <is>
-          <t>onsubmit -&gt; handlePosSale()</t>
-        </is>
-      </c>
-      <c r="C8" s="9" t="inlineStr">
+      <c r="B8" s="18" t="inlineStr">
+        <is>
+          <t>onSubmit -&gt; executeSale()</t>
+        </is>
+      </c>
+      <c r="C8" s="18" t="inlineStr">
         <is>
           <t>POST /api/sales</t>
         </is>
       </c>
-      <c r="D8" s="9" t="inlineStr">
+      <c r="D8" s="18" t="inlineStr">
         <is>
           <t>SaleService executes atomic transaction with rollback</t>
         </is>
       </c>
-      <c r="E8" s="9" t="inlineStr">
+      <c r="E8" s="18" t="inlineStr">
         <is>
           <t>UPDATE products; INSERT stock_transactions; INSERT sales</t>
         </is>
       </c>
-      <c r="F8" s="9" t="inlineStr">
-        <is>
-          <t>Inserts new row in sales receipt register; clears POS form.</t>
+      <c r="F8" s="18" t="inlineStr">
+        <is>
+          <t>Inserts record in sales register; triggers printable student receipt.</t>
         </is>
       </c>
     </row>
@@ -895,13 +1234,13 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:E6"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
-    <col width="48" customWidth="1" min="2" max="2"/>
-    <col width="48" customWidth="1" min="3" max="3"/>
-    <col width="48" customWidth="1" min="4" max="4"/>
-    <col width="48" customWidth="1" min="5" max="5"/>
+    <col width="55" customWidth="1" min="2" max="2"/>
+    <col width="55" customWidth="1" min="3" max="3"/>
+    <col width="55" customWidth="1" min="4" max="4"/>
+    <col width="55" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -912,109 +1251,109 @@
       </c>
     </row>
     <row r="2"/>
-    <row r="3" ht="25" customHeight="1">
-      <c r="A3" s="8" t="inlineStr">
+    <row r="3" ht="26" customHeight="1">
+      <c r="A3" s="15" t="inlineStr">
         <is>
           <t>Bug ID</t>
         </is>
       </c>
-      <c r="B3" s="8" t="inlineStr">
+      <c r="B3" s="15" t="inlineStr">
         <is>
           <t>Symptom / Error Encountered</t>
         </is>
       </c>
-      <c r="C3" s="8" t="inlineStr">
+      <c r="C3" s="15" t="inlineStr">
         <is>
           <t>Root Cause Analysis</t>
         </is>
       </c>
-      <c r="D3" s="8" t="inlineStr">
+      <c r="D3" s="15" t="inlineStr">
         <is>
           <t>Applied Resolution &amp; Code Fix</t>
         </is>
       </c>
-      <c r="E3" s="8" t="inlineStr">
+      <c r="E3" s="15" t="inlineStr">
         <is>
           <t>Verification &amp; Status</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="9" t="inlineStr">
+      <c r="A4" s="18" t="inlineStr">
         <is>
           <t>BUG-01</t>
         </is>
       </c>
-      <c r="B4" s="9" t="inlineStr">
-        <is>
-          <t>HTTP 404 Endpoint Not Found on /api/dashboard</t>
-        </is>
-      </c>
-      <c r="C4" s="9" t="inlineStr">
-        <is>
-          <t>Request routing checked /api/reports/dashboard but initial frontend called /api/dashboard.</t>
-        </is>
-      </c>
-      <c r="D4" s="9" t="inlineStr">
-        <is>
-          <t>Normalized API endpoint to /api/reports/dashboard across backend router and frontend client.</t>
-        </is>
-      </c>
-      <c r="E4" s="9" t="inlineStr">
-        <is>
-          <t>Verified via curl.exe; returns 200 OK with valid KPI JSON. [RESOLVED]</t>
+      <c r="B4" s="18" t="inlineStr">
+        <is>
+          <t>CORS policy blocked React frontend (:5173) requests to Java backend (:8080)</t>
+        </is>
+      </c>
+      <c r="C4" s="18" t="inlineStr">
+        <is>
+          <t>Java SimpleHttpServer did not return Access-Control-Allow-Origin response headers for cross-origin requests.</t>
+        </is>
+      </c>
+      <c r="D4" s="18" t="inlineStr">
+        <is>
+          <t>Added CORS header interceptor on SimpleHttpServer setting Access-Control-Allow-Origin: * and handling OPTIONS pre-flight.</t>
+        </is>
+      </c>
+      <c r="E4" s="18" t="inlineStr">
+        <is>
+          <t>Verified via curl.exe and browser console; 200 OK received without CORS warnings. [RESOLVED]</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="10" t="inlineStr">
+      <c r="A5" s="19" t="inlineStr">
         <is>
           <t>BUG-02</t>
         </is>
       </c>
-      <c r="B5" s="10" t="inlineStr">
+      <c r="B5" s="19" t="inlineStr">
         <is>
           <t>Overselling allowed when rapid sales executed concurrently</t>
         </is>
       </c>
-      <c r="C5" s="10" t="inlineStr">
+      <c r="C5" s="19" t="inlineStr">
         <is>
           <t>Stock check and stock decrement were two separate uncommitted database operations.</t>
         </is>
       </c>
-      <c r="D5" s="10" t="inlineStr">
+      <c r="D5" s="19" t="inlineStr">
         <is>
           <t>Enclosed stock check and decrement inside a single atomic transaction with setAutoCommit(false) and rollback().</t>
         </is>
       </c>
-      <c r="E5" s="10" t="inlineStr">
+      <c r="E5" s="19" t="inlineStr">
         <is>
           <t>Verified: Attempting to sell 100 with 6 in stock is immediately rejected. [RESOLVED]</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="9" t="inlineStr">
+      <c r="A6" s="18" t="inlineStr">
         <is>
           <t>BUG-03</t>
         </is>
       </c>
-      <c r="B6" s="9" t="inlineStr">
+      <c r="B6" s="18" t="inlineStr">
         <is>
           <t>Static frontend assets not accessible on port 8080</t>
         </is>
       </c>
-      <c r="C6" s="9" t="inlineStr">
+      <c r="C6" s="18" t="inlineStr">
         <is>
           <t>HttpServer originally only bound /api context, requiring a separate server for frontend.</t>
         </is>
       </c>
-      <c r="D6" s="9" t="inlineStr">
+      <c r="D6" s="18" t="inlineStr">
         <is>
           <t>Implemented StaticFileHandler on / context in SimpleHttpServer to serve HTML/CSS/JS directly.</t>
         </is>
       </c>
-      <c r="E6" s="9" t="inlineStr">
+      <c r="E6" s="18" t="inlineStr">
         <is>
           <t>Verified: Opening http://localhost:8080/ renders the full app directly from Java. [RESOLVED]</t>
         </is>
@@ -1032,12 +1371,12 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:D7"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
-    <col width="48" customWidth="1" min="1" max="1"/>
+    <col width="50" customWidth="1" min="1" max="1"/>
     <col width="25" customWidth="1" min="2" max="2"/>
     <col width="29" customWidth="1" min="3" max="3"/>
-    <col width="48" customWidth="1" min="4" max="4"/>
+    <col width="55" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1048,113 +1387,113 @@
       </c>
     </row>
     <row r="2"/>
-    <row r="3" ht="25" customHeight="1">
-      <c r="A3" s="8" t="inlineStr">
+    <row r="3" ht="26" customHeight="1">
+      <c r="A3" s="15" t="inlineStr">
         <is>
           <t>Time Interval</t>
         </is>
       </c>
-      <c r="B3" s="8" t="inlineStr">
+      <c r="B3" s="15" t="inlineStr">
         <is>
           <t>Speaker Name &amp; Reg No</t>
         </is>
       </c>
-      <c r="C3" s="8" t="inlineStr">
+      <c r="C3" s="15" t="inlineStr">
         <is>
           <t>Role</t>
         </is>
       </c>
-      <c r="D3" s="8" t="inlineStr">
+      <c r="D3" s="15" t="inlineStr">
         <is>
           <t>Viva Pitch Script Content &amp; Examiner Talking Points</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="9" t="inlineStr">
+      <c r="A4" s="18" t="inlineStr">
         <is>
           <t>0:00 - 0:45</t>
         </is>
       </c>
-      <c r="B4" s="9" t="inlineStr">
+      <c r="B4" s="18" t="inlineStr">
         <is>
           <t>Nikhila V (44731059)</t>
         </is>
       </c>
-      <c r="C4" s="9" t="inlineStr">
+      <c r="C4" s="18" t="inlineStr">
         <is>
           <t>Lead Architect</t>
         </is>
       </c>
-      <c r="D4" s="9" t="inlineStr">
-        <is>
-          <t>Good morning respected examiners. Our project is the Smart Stationery Inventory Management System. Stationery retail faces unique problems: managing hundreds of small SKUs in paper registers leads to human errors, untracked damaged items, and severe stock-outs during back-to-school exam rushes. To solve this, we architected a lightweight, framework-independent 3-tier solution using Core Java 21, plain JDBC, and Vanilla Web technologies.</t>
+      <c r="D4" s="18" t="inlineStr">
+        <is>
+          <t>Good morning respected examiners. We represent Sathyabama Institute of Science and Technology (SIST), Department of CSE AI, Batch 2023-2027 Section A4. Our capstone project is the Smart Stationery Inventory Management System. Stationery retail faces unique problems: managing hundreds of small SKUs in paper registers leads to human math errors, untracked damaged goods, and severe stock-outs during back-to-school exam rushes. To solve this, we architected a robust 3-tier solution using Core Java 21, plain JDBC, MySQL 8.0, and modern React 19 with a Vanilla Web companion.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="10" t="inlineStr">
+      <c r="A5" s="19" t="inlineStr">
         <is>
           <t>0:45 - 1:45</t>
         </is>
       </c>
-      <c r="B5" s="10" t="inlineStr">
+      <c r="B5" s="19" t="inlineStr">
         <is>
           <t>Zaid Basha (44731049)</t>
         </is>
       </c>
-      <c r="C5" s="10" t="inlineStr">
+      <c r="C5" s="19" t="inlineStr">
         <is>
           <t>Backend &amp; DB Specialist</t>
         </is>
       </c>
-      <c r="D5" s="10" t="inlineStr">
-        <is>
-          <t>On the backend, we deliberately avoided Spring Boot and Hibernate to demonstrate mastery over core computer science principles. Our Java server uses standard library HttpServer with Java 21 Virtual Threads and raw JDBC PreparedStatements. In MySQL, our 5 tables in 3NF enforce non-negative stock (CHECK quantity &gt;= 0). For POS billing, we coordinate an atomic 3-way transaction ensuring stock decrements, sales receipts, and audit ledger entries succeed together or rollback completely.</t>
+      <c r="D5" s="19" t="inlineStr">
+        <is>
+          <t>On the backend, we demonstrate mastery over core computer science principles without relying on bulky frameworks. Our Java backend uses standard library HttpServer with Java 21 Virtual Threads and raw JDBC PreparedStatements for 100% SQL injection immunity. In MySQL, our 5 tables in 3NF enforce non-negative stock (CHECK quantity &gt;= 0). For POS billing, we coordinate an atomic 3-way transaction ensuring stock decrements, customer receipts, and audit ledger entries succeed together or rollback completely.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="9" t="inlineStr">
+      <c r="A6" s="18" t="inlineStr">
         <is>
           <t>1:45 - 2:30</t>
         </is>
       </c>
-      <c r="B6" s="9" t="inlineStr">
+      <c r="B6" s="18" t="inlineStr">
         <is>
           <t>Nikhila V (44731059)</t>
         </is>
       </c>
-      <c r="C6" s="9" t="inlineStr">
+      <c r="C6" s="18" t="inlineStr">
         <is>
           <t>Lead Architect &amp; Frontend</t>
         </is>
       </c>
-      <c r="D6" s="9" t="inlineStr">
-        <is>
-          <t>On the frontend, we used pure HTML5, CSS3, and Vanilla JavaScript with zero external libraries. As you can see on the live dashboard on port 8080, when stock drops below the threshold, the system displays an amber LOW STOCK badge and calculates the exact suggested reorder units using: (Reorder Point * 2) - Current Qty. We also built a pure client-side CSV generator allowing 1-click spreadsheet export for vendor orders.</t>
+      <c r="D6" s="18" t="inlineStr">
+        <is>
+          <t>On the frontend, we built both a sleek React 19 application running on port 5173 with role-based authentication (admin, staff1, staff2) and a pure Vanilla HTML5/CSS3 interface. As you can see on the live dashboard, when stock drops below the safety threshold, the system displays an amber LOW STOCK badge and calculates the exact suggested reorder units: (Reorder Point * 2) - Current Qty. We also built client-side CSV export allowing 1-click vendor order spreadsheets.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="10" t="inlineStr">
+      <c r="A7" s="19" t="inlineStr">
         <is>
           <t>2:30 - 3:00</t>
         </is>
       </c>
-      <c r="B7" s="10" t="inlineStr">
+      <c r="B7" s="19" t="inlineStr">
         <is>
           <t>Team (Nikhila &amp; Zaid)</t>
         </is>
       </c>
-      <c r="C7" s="10" t="inlineStr">
+      <c r="C7" s="19" t="inlineStr">
         <is>
           <t>Joint Conclusion</t>
         </is>
       </c>
-      <c r="D7" s="10" t="inlineStr">
-        <is>
-          <t>Every module has passed 100% of our acceptance test suites, and the entire system launches in 1-click using run.bat. We are now pleased to demonstrate the live application running on localhost:8080 and welcome any questions from the panel.</t>
+      <c r="D7" s="19" t="inlineStr">
+        <is>
+          <t>Every single module has passed 100% of our acceptance test suites. The code is version-controlled on GitHub across main, dev, and feature branches, and the system launches in 1-click using run.bat. We are pleased to demonstrate the live application running on http://127.0.0.1:5173 and http://localhost:8080/api and welcome any questions from the panel.</t>
         </is>
       </c>
     </row>
@@ -1170,11 +1509,11 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:C14"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
-    <col width="48" customWidth="1" min="1" max="1"/>
+    <col width="55" customWidth="1" min="1" max="1"/>
     <col width="36" customWidth="1" min="2" max="2"/>
-    <col width="48" customWidth="1" min="3" max="3"/>
+    <col width="55" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1185,205 +1524,205 @@
       </c>
     </row>
     <row r="2"/>
-    <row r="3" ht="25" customHeight="1">
-      <c r="A3" s="8" t="inlineStr">
+    <row r="3" ht="26" customHeight="1">
+      <c r="A3" s="15" t="inlineStr">
         <is>
           <t>Section</t>
         </is>
       </c>
-      <c r="B3" s="8" t="inlineStr">
+      <c r="B3" s="15" t="inlineStr">
         <is>
           <t>Parameter</t>
         </is>
       </c>
-      <c r="C3" s="8" t="inlineStr">
+      <c r="C3" s="15" t="inlineStr">
         <is>
           <t>Detailed Academic Specification</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="9" t="inlineStr">
+      <c r="A4" s="18" t="inlineStr">
         <is>
           <t>Target Persona 1</t>
         </is>
       </c>
-      <c r="B4" s="9" t="inlineStr">
+      <c r="B4" s="18" t="inlineStr">
         <is>
           <t>Suresh Sharma (Store Owner)</t>
         </is>
       </c>
-      <c r="C4" s="9" t="inlineStr">
+      <c r="C4" s="18" t="inlineStr">
         <is>
           <t>Needs automated reorder warnings and instant inventory valuation by category to prevent lost sales during back-to-school surges.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="10" t="inlineStr">
+      <c r="A5" s="19" t="inlineStr">
         <is>
           <t>Target Persona 2</t>
         </is>
       </c>
-      <c r="B5" s="10" t="inlineStr">
+      <c r="B5" s="19" t="inlineStr">
         <is>
           <t>Priya Patel (Cashier / Staff)</t>
         </is>
       </c>
-      <c r="C5" s="10" t="inlineStr">
+      <c r="C5" s="19" t="inlineStr">
         <is>
           <t>Requires high-speed POS billing with automatic stock decrements and overselling prevention to speed up student checkout.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="9" t="inlineStr">
+      <c r="A6" s="18" t="inlineStr">
         <is>
           <t>Problem Statement</t>
         </is>
       </c>
-      <c r="B6" s="9" t="inlineStr">
+      <c r="B6" s="18" t="inlineStr">
         <is>
           <t>Stationery Retail Inefficiencies</t>
         </is>
       </c>
-      <c r="C6" s="9" t="inlineStr">
+      <c r="C6" s="18" t="inlineStr">
         <is>
           <t>Stationery stores manage hundreds of low-cost SKUs in paper notebooks. Manual entries cause math errors, untracked damage write-offs, and stock-outs.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="10" t="inlineStr">
+      <c r="A7" s="19" t="inlineStr">
         <is>
           <t>MoSCoW - Must Have</t>
         </is>
       </c>
-      <c r="B7" s="10" t="inlineStr">
+      <c r="B7" s="19" t="inlineStr">
         <is>
           <t>Core Inventory &amp; POS</t>
         </is>
       </c>
-      <c r="C7" s="10" t="inlineStr">
+      <c r="C7" s="19" t="inlineStr">
         <is>
           <t>Real-time stock tracking with bin locations, non-negative stock constraint, atomic POS sales, and immutable audit ledger.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="9" t="inlineStr">
+      <c r="A8" s="18" t="inlineStr">
         <is>
           <t>MoSCoW - Should Have</t>
         </is>
       </c>
-      <c r="B8" s="9" t="inlineStr">
+      <c r="B8" s="18" t="inlineStr">
         <is>
           <t>KPIs &amp; CSV Export</t>
         </is>
       </c>
-      <c r="C8" s="9" t="inlineStr">
+      <c r="C8" s="18" t="inlineStr">
         <is>
           <t>Executive store dashboard with 4 metric cards, and 1-click client-side CSV spreadsheet generation.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="10" t="inlineStr">
+      <c r="A9" s="19" t="inlineStr">
         <is>
           <t>MoSCoW - Could Have</t>
         </is>
       </c>
-      <c r="B9" s="10" t="inlineStr">
+      <c r="B9" s="19" t="inlineStr">
         <is>
           <t>Shelf Bin Indexing</t>
         </is>
       </c>
-      <c r="C9" s="10" t="inlineStr">
+      <c r="C9" s="19" t="inlineStr">
         <is>
           <t>Shelf bin tracking (e.g. A01, B02) to streamline stock retrieval in retail aisles.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="9" t="inlineStr">
+      <c r="A10" s="18" t="inlineStr">
         <is>
           <t>MoSCoW - Won't Have</t>
         </is>
       </c>
-      <c r="B10" s="9" t="inlineStr">
+      <c r="B10" s="18" t="inlineStr">
         <is>
           <t>Biometrics / E-commerce</t>
         </is>
       </c>
-      <c r="C10" s="9" t="inlineStr">
+      <c r="C10" s="18" t="inlineStr">
         <is>
           <t>Deferred to commercial enterprise release.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="10" t="inlineStr">
+      <c r="A11" s="19" t="inlineStr">
         <is>
           <t>NFR-1</t>
         </is>
       </c>
-      <c r="B11" s="10" t="inlineStr">
+      <c r="B11" s="19" t="inlineStr">
         <is>
           <t>Performance</t>
         </is>
       </c>
-      <c r="C11" s="10" t="inlineStr">
+      <c r="C11" s="19" t="inlineStr">
         <is>
           <t>Local REST endpoints must respond in &lt; 30ms via Java 21 lightweight Virtual Threads.</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="9" t="inlineStr">
+      <c r="A12" s="18" t="inlineStr">
         <is>
           <t>NFR-2</t>
         </is>
       </c>
-      <c r="B12" s="9" t="inlineStr">
+      <c r="B12" s="18" t="inlineStr">
         <is>
           <t>Security</t>
         </is>
       </c>
-      <c r="C12" s="9" t="inlineStr">
+      <c r="C12" s="18" t="inlineStr">
         <is>
           <t>100% Parameterized SQL queries using JDBC PreparedStatement to guarantee total SQL injection immunity.</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="10" t="inlineStr">
+      <c r="A13" s="19" t="inlineStr">
         <is>
           <t>NFR-3</t>
         </is>
       </c>
-      <c r="B13" s="10" t="inlineStr">
+      <c r="B13" s="19" t="inlineStr">
         <is>
           <t>Data Integrity</t>
         </is>
       </c>
-      <c r="C13" s="10" t="inlineStr">
+      <c r="C13" s="19" t="inlineStr">
         <is>
           <t>Normalized 3NF MySQL schema with ACID transaction isolation and CHECK (quantity &gt;= 0).</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="9" t="inlineStr">
+      <c r="A14" s="18" t="inlineStr">
         <is>
           <t>NFR-4</t>
         </is>
       </c>
-      <c r="B14" s="9" t="inlineStr">
+      <c r="B14" s="18" t="inlineStr">
         <is>
           <t>Explainability</t>
         </is>
       </c>
-      <c r="C14" s="9" t="inlineStr">
+      <c r="C14" s="18" t="inlineStr">
         <is>
           <t>Pure Java SE and Vanilla JS with zero framework abstractions for student viva defense.</t>
         </is>
@@ -1401,13 +1740,13 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:E9"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
-    <col width="48" customWidth="1" min="1" max="1"/>
+    <col width="54" customWidth="1" min="1" max="1"/>
     <col width="17" customWidth="1" min="2" max="2"/>
-    <col width="48" customWidth="1" min="3" max="3"/>
-    <col width="48" customWidth="1" min="4" max="4"/>
-    <col width="48" customWidth="1" min="5" max="5"/>
+    <col width="51" customWidth="1" min="3" max="3"/>
+    <col width="55" customWidth="1" min="4" max="4"/>
+    <col width="55" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1418,190 +1757,190 @@
       </c>
     </row>
     <row r="2"/>
-    <row r="3" ht="25" customHeight="1">
-      <c r="A3" s="8" t="inlineStr">
+    <row r="3" ht="26" customHeight="1">
+      <c r="A3" s="15" t="inlineStr">
         <is>
           <t>Story ID</t>
         </is>
       </c>
-      <c r="B3" s="8" t="inlineStr">
+      <c r="B3" s="15" t="inlineStr">
         <is>
           <t>Role</t>
         </is>
       </c>
-      <c r="C3" s="8" t="inlineStr">
+      <c r="C3" s="15" t="inlineStr">
         <is>
           <t>User Story Description</t>
         </is>
       </c>
-      <c r="D3" s="8" t="inlineStr">
+      <c r="D3" s="15" t="inlineStr">
         <is>
           <t>Scenario 1 (Given / When / Then)</t>
         </is>
       </c>
-      <c r="E3" s="8" t="inlineStr">
+      <c r="E3" s="15" t="inlineStr">
         <is>
           <t>Scenario 2 (Given / When / Then)</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="9" t="inlineStr">
+      <c r="A4" s="18" t="inlineStr">
         <is>
           <t>US-01</t>
         </is>
       </c>
-      <c r="B4" s="9" t="inlineStr">
+      <c r="B4" s="18" t="inlineStr">
         <is>
           <t>Store Manager</t>
         </is>
       </c>
-      <c r="C4" s="9" t="inlineStr">
+      <c r="C4" s="18" t="inlineStr">
         <is>
           <t>Register new products with unique SKU</t>
         </is>
       </c>
-      <c r="D4" s="9" t="inlineStr">
+      <c r="D4" s="18" t="inlineStr">
         <is>
           <t>Given valid fields -&gt; When saved -&gt; Then product created with IN STOCK badge.</t>
         </is>
       </c>
-      <c r="E4" s="9" t="inlineStr">
+      <c r="E4" s="18" t="inlineStr">
         <is>
           <t>Given existing SKU 'PEN001' -&gt; When saved -&gt; Then HTTP 409 Conflict returned.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="10" t="inlineStr">
+      <c r="A5" s="19" t="inlineStr">
         <is>
           <t>US-02</t>
         </is>
       </c>
-      <c r="B5" s="10" t="inlineStr">
+      <c r="B5" s="19" t="inlineStr">
         <is>
           <t>Store Manager</t>
         </is>
       </c>
-      <c r="C5" s="10" t="inlineStr">
+      <c r="C5" s="19" t="inlineStr">
         <is>
           <t>Automatic low-stock warnings &amp; reorder quantity</t>
         </is>
       </c>
-      <c r="D5" s="10" t="inlineStr">
+      <c r="D5" s="19" t="inlineStr">
         <is>
           <t>Given qty &lt;= reorder -&gt; When queried -&gt; Then status is LOW STOCK and suggested order is calculated.</t>
         </is>
       </c>
-      <c r="E5" s="10" t="inlineStr">
+      <c r="E5" s="19" t="inlineStr">
         <is>
           <t>Given qty == 0 -&gt; When queried -&gt; Then status is OUT OF STOCK with red badge.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="9" t="inlineStr">
+      <c r="A6" s="18" t="inlineStr">
         <is>
           <t>US-03</t>
         </is>
       </c>
-      <c r="B6" s="9" t="inlineStr">
+      <c r="B6" s="18" t="inlineStr">
         <is>
           <t>Store Cashier</t>
         </is>
       </c>
-      <c r="C6" s="9" t="inlineStr">
+      <c r="C6" s="18" t="inlineStr">
         <is>
           <t>Execute atomic POS customer billing</t>
         </is>
       </c>
-      <c r="D6" s="9" t="inlineStr">
+      <c r="D6" s="18" t="inlineStr">
         <is>
           <t>Given 150 pens in stock -&gt; When sell 5 units -&gt; Then stock drops to 145 and sale is recorded.</t>
         </is>
       </c>
-      <c r="E6" s="9" t="inlineStr">
+      <c r="E6" s="18" t="inlineStr">
         <is>
           <t>Given 6 staplers in stock -&gt; When sell 10 units -&gt; Then transaction rolls back with error.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="10" t="inlineStr">
+      <c r="A7" s="19" t="inlineStr">
         <is>
           <t>US-04</t>
         </is>
       </c>
-      <c r="B7" s="10" t="inlineStr">
+      <c r="B7" s="19" t="inlineStr">
         <is>
           <t>Storekeeper</t>
         </is>
       </c>
-      <c r="C7" s="10" t="inlineStr">
+      <c r="C7" s="19" t="inlineStr">
         <is>
           <t>Record inward delivery shipments</t>
         </is>
       </c>
-      <c r="D7" s="10" t="inlineStr">
+      <c r="D7" s="19" t="inlineStr">
         <is>
           <t>Given item with 8 units -&gt; When restock +50 units -&gt; Then stock becomes 58 and status changes to IN STOCK.</t>
         </is>
       </c>
-      <c r="E7" s="10" t="inlineStr">
+      <c r="E7" s="19" t="inlineStr">
         <is>
           <t>Given invalid product -&gt; When restock -&gt; Then rejected with HTTP 400.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="9" t="inlineStr">
+      <c r="A8" s="18" t="inlineStr">
         <is>
           <t>US-05</t>
         </is>
       </c>
-      <c r="B8" s="9" t="inlineStr">
+      <c r="B8" s="18" t="inlineStr">
         <is>
           <t>Storekeeper</t>
         </is>
       </c>
-      <c r="C8" s="9" t="inlineStr">
+      <c r="C8" s="18" t="inlineStr">
         <is>
           <t>Write off damaged goods with audit reason</t>
         </is>
       </c>
-      <c r="D8" s="9" t="inlineStr">
+      <c r="D8" s="18" t="inlineStr">
         <is>
           <t>Given 20 markers -&gt; When write off 2 damaged units -&gt; Then stock drops to 18 and ledger logs DAMAGED.</t>
         </is>
       </c>
-      <c r="E8" s="9" t="inlineStr">
+      <c r="E8" s="18" t="inlineStr">
         <is>
           <t>Given 5 units in stock -&gt; When attempt 10 damaged -&gt; Then rejected with insufficient stock.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="10" t="inlineStr">
+      <c r="A9" s="19" t="inlineStr">
         <is>
           <t>US-06</t>
         </is>
       </c>
-      <c r="B9" s="10" t="inlineStr">
+      <c r="B9" s="19" t="inlineStr">
         <is>
           <t>Store Owner</t>
         </is>
       </c>
-      <c r="C9" s="10" t="inlineStr">
+      <c r="C9" s="19" t="inlineStr">
         <is>
           <t>View category valuations &amp; download CSV</t>
         </is>
       </c>
-      <c r="D9" s="10" t="inlineStr">
+      <c r="D9" s="19" t="inlineStr">
         <is>
           <t>Given items in Pens category -&gt; When report loaded -&gt; Then category valuation is summed correctly.</t>
         </is>
       </c>
-      <c r="E9" s="10" t="inlineStr">
+      <c r="E9" s="19" t="inlineStr">
         <is>
           <t>Given report on screen -&gt; When click Download CSV -&gt; Then .csv file is downloaded.</t>
         </is>
@@ -1619,14 +1958,14 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:F6"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
-    <col width="48" customWidth="1" min="1" max="1"/>
+    <col width="50" customWidth="1" min="1" max="1"/>
     <col width="28" customWidth="1" min="2" max="2"/>
     <col width="15" customWidth="1" min="3" max="3"/>
-    <col width="45" customWidth="1" min="4" max="4"/>
-    <col width="48" customWidth="1" min="5" max="5"/>
-    <col width="48" customWidth="1" min="6" max="6"/>
+    <col width="47" customWidth="1" min="4" max="4"/>
+    <col width="55" customWidth="1" min="5" max="5"/>
+    <col width="55" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1637,131 +1976,131 @@
       </c>
     </row>
     <row r="2"/>
-    <row r="3" ht="25" customHeight="1">
-      <c r="A3" s="8" t="inlineStr">
+    <row r="3" ht="26" customHeight="1">
+      <c r="A3" s="15" t="inlineStr">
         <is>
           <t>Tier</t>
         </is>
       </c>
-      <c r="B3" s="8" t="inlineStr">
+      <c r="B3" s="15" t="inlineStr">
         <is>
           <t>Layer Name</t>
         </is>
       </c>
-      <c r="C3" s="8" t="inlineStr">
+      <c r="C3" s="15" t="inlineStr">
         <is>
           <t>Port</t>
         </is>
       </c>
-      <c r="D3" s="8" t="inlineStr">
+      <c r="D3" s="15" t="inlineStr">
         <is>
           <t>Technology</t>
         </is>
       </c>
-      <c r="E3" s="8" t="inlineStr">
+      <c r="E3" s="15" t="inlineStr">
         <is>
           <t>Component Responsibilities</t>
         </is>
       </c>
-      <c r="F3" s="8" t="inlineStr">
+      <c r="F3" s="15" t="inlineStr">
         <is>
           <t>Data Flow &amp; Security</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="9" t="inlineStr">
+      <c r="A4" s="18" t="inlineStr">
         <is>
           <t>Tier 1</t>
         </is>
       </c>
-      <c r="B4" s="9" t="inlineStr">
+      <c r="B4" s="18" t="inlineStr">
         <is>
           <t>Presentation Tier</t>
         </is>
       </c>
-      <c r="C4" s="9" t="inlineStr">
-        <is>
-          <t>5500 / 8080</t>
-        </is>
-      </c>
-      <c r="D4" s="9" t="inlineStr">
-        <is>
-          <t>HTML5, CSS3, Vanilla JS (ES6+)</t>
-        </is>
-      </c>
-      <c r="E4" s="9" t="inlineStr">
-        <is>
-          <t>Renders dashboard, responsive product catalog, modal forms, and POS checkout interface.</t>
-        </is>
-      </c>
-      <c r="F4" s="9" t="inlineStr">
-        <is>
-          <t>Sends async fetch() JSON requests to :8080/api. Displays real-time DOM updates.</t>
+      <c r="C4" s="18" t="inlineStr">
+        <is>
+          <t>5173 / 8080</t>
+        </is>
+      </c>
+      <c r="D4" s="18" t="inlineStr">
+        <is>
+          <t>React 19 (Vite) &amp; HTML5/CSS3/Vanilla JS</t>
+        </is>
+      </c>
+      <c r="E4" s="18" t="inlineStr">
+        <is>
+          <t>Renders responsive dashboard, product catalog, inventory table, POS billing modal, and role-based login (admin, staff1, staff2).</t>
+        </is>
+      </c>
+      <c r="F4" s="18" t="inlineStr">
+        <is>
+          <t>Sends asynchronous fetch() JSON requests to :8080/api. Displays real-time DOM/React state updates.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="10" t="inlineStr">
+      <c r="A5" s="19" t="inlineStr">
         <is>
           <t>Tier 2</t>
         </is>
       </c>
-      <c r="B5" s="10" t="inlineStr">
+      <c r="B5" s="19" t="inlineStr">
         <is>
           <t>Application / Logic Tier</t>
         </is>
       </c>
-      <c r="C5" s="10" t="inlineStr">
+      <c r="C5" s="19" t="inlineStr">
         <is>
           <t>8080</t>
         </is>
       </c>
-      <c r="D5" s="10" t="inlineStr">
-        <is>
-          <t>Java 21 SE (HttpServer / Virtual Threads)</t>
-        </is>
-      </c>
-      <c r="E5" s="10" t="inlineStr">
-        <is>
-          <t>Dispatches requests, validates business rules, computes reorder formulas, and enforces ACID transactions.</t>
-        </is>
-      </c>
-      <c r="F5" s="10" t="inlineStr">
-        <is>
-          <t>Communicates with MySQL using thread-safe plain JDBC PreparedStatement connection pool.</t>
+      <c r="D5" s="19" t="inlineStr">
+        <is>
+          <t>Core Java 21 (HttpServer / Virtual Threads)</t>
+        </is>
+      </c>
+      <c r="E5" s="19" t="inlineStr">
+        <is>
+          <t>Dispatches REST API routes, validates input parameters, computes reorder formulas, and coordinates atomic transactions.</t>
+        </is>
+      </c>
+      <c r="F5" s="19" t="inlineStr">
+        <is>
+          <t>Communicates with MySQL using thread-safe plain JDBC PreparedStatement connection factory with zero framework overhead.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="9" t="inlineStr">
+      <c r="A6" s="18" t="inlineStr">
         <is>
           <t>Tier 3</t>
         </is>
       </c>
-      <c r="B6" s="9" t="inlineStr">
+      <c r="B6" s="18" t="inlineStr">
         <is>
           <t>Data Persistence Tier</t>
         </is>
       </c>
-      <c r="C6" s="9" t="inlineStr">
+      <c r="C6" s="18" t="inlineStr">
         <is>
           <t>3306</t>
         </is>
       </c>
-      <c r="D6" s="9" t="inlineStr">
-        <is>
-          <t>MySQL Server 8.0 (InnoDB)</t>
-        </is>
-      </c>
-      <c r="E6" s="9" t="inlineStr">
-        <is>
-          <t>Stores 5 normalized 3NF relational tables, enforces foreign keys and non-negative constraints.</t>
-        </is>
-      </c>
-      <c r="F6" s="9" t="inlineStr">
-        <is>
-          <t>Executes parameterized SQL queries with row-level locking and transaction rollback on error.</t>
+      <c r="D6" s="18" t="inlineStr">
+        <is>
+          <t>MySQL Server 8.0 (InnoDB Engine)</t>
+        </is>
+      </c>
+      <c r="E6" s="18" t="inlineStr">
+        <is>
+          <t>Stores 5 normalized 3NF relational tables, enforces foreign key constraints and non-negative quantity check.</t>
+        </is>
+      </c>
+      <c r="F6" s="18" t="inlineStr">
+        <is>
+          <t>Executes parameterized SQL queries with row-level locking, ACID guarantee, and transaction rollback on error.</t>
         </is>
       </c>
     </row>
@@ -1777,7 +2116,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:F32"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="45" customWidth="1" min="1" max="1"/>
     <col width="20" customWidth="1" min="2" max="2"/>
@@ -1795,961 +2134,961 @@
       </c>
     </row>
     <row r="2"/>
-    <row r="3" ht="25" customHeight="1">
-      <c r="A3" s="8" t="inlineStr">
+    <row r="3" ht="26" customHeight="1">
+      <c r="A3" s="15" t="inlineStr">
         <is>
           <t>Table Name</t>
         </is>
       </c>
-      <c r="B3" s="8" t="inlineStr">
+      <c r="B3" s="15" t="inlineStr">
         <is>
           <t>Column Name</t>
         </is>
       </c>
-      <c r="C3" s="8" t="inlineStr">
+      <c r="C3" s="15" t="inlineStr">
         <is>
           <t>Data Type</t>
         </is>
       </c>
-      <c r="D3" s="8" t="inlineStr">
+      <c r="D3" s="15" t="inlineStr">
         <is>
           <t>Constraint / Key</t>
         </is>
       </c>
-      <c r="E3" s="8" t="inlineStr">
+      <c r="E3" s="15" t="inlineStr">
         <is>
           <t>Default</t>
         </is>
       </c>
-      <c r="F3" s="8" t="inlineStr">
+      <c r="F3" s="15" t="inlineStr">
         <is>
           <t>Description &amp; Purpose</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="11" t="inlineStr">
+      <c r="A4" s="20" t="inlineStr">
         <is>
           <t>categories</t>
         </is>
       </c>
-      <c r="B4" s="11" t="inlineStr">
+      <c r="B4" s="20" t="inlineStr">
         <is>
           <t>category_id</t>
         </is>
       </c>
-      <c r="C4" s="11" t="inlineStr">
+      <c r="C4" s="20" t="inlineStr">
         <is>
           <t>INT</t>
         </is>
       </c>
-      <c r="D4" s="11" t="inlineStr">
+      <c r="D4" s="20" t="inlineStr">
         <is>
           <t>PRIMARY KEY, AUTO_INCREMENT</t>
         </is>
       </c>
-      <c r="E4" s="11" t="inlineStr">
+      <c r="E4" s="20" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="F4" s="11" t="inlineStr">
+      <c r="F4" s="20" t="inlineStr">
         <is>
           <t>Unique category identifier</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="12" t="inlineStr">
+      <c r="A5" s="21" t="inlineStr">
         <is>
           <t>categories</t>
         </is>
       </c>
-      <c r="B5" s="12" t="inlineStr">
+      <c r="B5" s="21" t="inlineStr">
         <is>
           <t>category_name</t>
         </is>
       </c>
-      <c r="C5" s="12" t="inlineStr">
+      <c r="C5" s="21" t="inlineStr">
         <is>
           <t>VARCHAR(100)</t>
         </is>
       </c>
-      <c r="D5" s="12" t="inlineStr">
+      <c r="D5" s="21" t="inlineStr">
         <is>
           <t>UNIQUE, NOT NULL</t>
         </is>
       </c>
-      <c r="E5" s="12" t="inlineStr">
+      <c r="E5" s="21" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="F5" s="12" t="inlineStr">
+      <c r="F5" s="21" t="inlineStr">
         <is>
           <t>Name of category (Pens, Notebooks, etc.)</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="11" t="inlineStr">
+      <c r="A6" s="20" t="inlineStr">
         <is>
           <t>suppliers</t>
         </is>
       </c>
-      <c r="B6" s="11" t="inlineStr">
+      <c r="B6" s="20" t="inlineStr">
         <is>
           <t>supplier_id</t>
         </is>
       </c>
-      <c r="C6" s="11" t="inlineStr">
+      <c r="C6" s="20" t="inlineStr">
         <is>
           <t>INT</t>
         </is>
       </c>
-      <c r="D6" s="11" t="inlineStr">
+      <c r="D6" s="20" t="inlineStr">
         <is>
           <t>PRIMARY KEY, AUTO_INCREMENT</t>
         </is>
       </c>
-      <c r="E6" s="11" t="inlineStr">
+      <c r="E6" s="20" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="F6" s="11" t="inlineStr">
+      <c r="F6" s="20" t="inlineStr">
         <is>
           <t>Unique supplier vendor identifier</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="12" t="inlineStr">
+      <c r="A7" s="21" t="inlineStr">
         <is>
           <t>suppliers</t>
         </is>
       </c>
-      <c r="B7" s="12" t="inlineStr">
+      <c r="B7" s="21" t="inlineStr">
         <is>
           <t>supplier_name</t>
         </is>
       </c>
-      <c r="C7" s="12" t="inlineStr">
+      <c r="C7" s="21" t="inlineStr">
         <is>
           <t>VARCHAR(150)</t>
         </is>
       </c>
-      <c r="D7" s="12" t="inlineStr">
+      <c r="D7" s="21" t="inlineStr">
         <is>
           <t>NOT NULL</t>
         </is>
       </c>
-      <c r="E7" s="12" t="inlineStr">
+      <c r="E7" s="21" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="F7" s="12" t="inlineStr">
+      <c r="F7" s="21" t="inlineStr">
         <is>
           <t>Supplier business/company name</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="11" t="inlineStr">
+      <c r="A8" s="20" t="inlineStr">
         <is>
           <t>suppliers</t>
         </is>
       </c>
-      <c r="B8" s="11" t="inlineStr">
+      <c r="B8" s="20" t="inlineStr">
         <is>
           <t>contact_person</t>
         </is>
       </c>
-      <c r="C8" s="11" t="inlineStr">
+      <c r="C8" s="20" t="inlineStr">
         <is>
           <t>VARCHAR(100)</t>
         </is>
       </c>
-      <c r="D8" s="11" t="inlineStr">
+      <c r="D8" s="20" t="inlineStr">
         <is>
           <t>NULLABLE</t>
         </is>
       </c>
-      <c r="E8" s="11" t="inlineStr">
+      <c r="E8" s="20" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="F8" s="11" t="inlineStr">
+      <c r="F8" s="20" t="inlineStr">
         <is>
           <t>Vendor representative contact name</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="12" t="inlineStr">
+      <c r="A9" s="21" t="inlineStr">
         <is>
           <t>suppliers</t>
         </is>
       </c>
-      <c r="B9" s="12" t="inlineStr">
+      <c r="B9" s="21" t="inlineStr">
         <is>
           <t>phone</t>
         </is>
       </c>
-      <c r="C9" s="12" t="inlineStr">
+      <c r="C9" s="21" t="inlineStr">
         <is>
           <t>VARCHAR(20)</t>
         </is>
       </c>
-      <c r="D9" s="12" t="inlineStr">
+      <c r="D9" s="21" t="inlineStr">
         <is>
           <t>NULLABLE</t>
         </is>
       </c>
-      <c r="E9" s="12" t="inlineStr">
+      <c r="E9" s="21" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="F9" s="12" t="inlineStr">
+      <c r="F9" s="21" t="inlineStr">
         <is>
           <t>Supplier contact telephone/mobile</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="11" t="inlineStr">
+      <c r="A10" s="20" t="inlineStr">
         <is>
           <t>suppliers</t>
         </is>
       </c>
-      <c r="B10" s="11" t="inlineStr">
+      <c r="B10" s="20" t="inlineStr">
         <is>
           <t>email</t>
         </is>
       </c>
-      <c r="C10" s="11" t="inlineStr">
+      <c r="C10" s="20" t="inlineStr">
         <is>
           <t>VARCHAR(100)</t>
         </is>
       </c>
-      <c r="D10" s="11" t="inlineStr">
+      <c r="D10" s="20" t="inlineStr">
         <is>
           <t>NULLABLE</t>
         </is>
       </c>
-      <c r="E10" s="11" t="inlineStr">
+      <c r="E10" s="20" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="F10" s="11" t="inlineStr">
+      <c r="F10" s="20" t="inlineStr">
         <is>
           <t>Supplier order communication email</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="12" t="inlineStr">
+      <c r="A11" s="21" t="inlineStr">
         <is>
           <t>suppliers</t>
         </is>
       </c>
-      <c r="B11" s="12" t="inlineStr">
+      <c r="B11" s="21" t="inlineStr">
         <is>
           <t>address</t>
         </is>
       </c>
-      <c r="C11" s="12" t="inlineStr">
+      <c r="C11" s="21" t="inlineStr">
         <is>
           <t>TEXT</t>
         </is>
       </c>
-      <c r="D11" s="12" t="inlineStr">
+      <c r="D11" s="21" t="inlineStr">
         <is>
           <t>NULLABLE</t>
         </is>
       </c>
-      <c r="E11" s="12" t="inlineStr">
+      <c r="E11" s="21" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="F11" s="12" t="inlineStr">
+      <c r="F11" s="21" t="inlineStr">
         <is>
           <t>Warehouse dispatch address</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="11" t="inlineStr">
+      <c r="A12" s="20" t="inlineStr">
         <is>
           <t>products</t>
         </is>
       </c>
-      <c r="B12" s="11" t="inlineStr">
+      <c r="B12" s="20" t="inlineStr">
         <is>
           <t>product_id</t>
         </is>
       </c>
-      <c r="C12" s="11" t="inlineStr">
+      <c r="C12" s="20" t="inlineStr">
         <is>
           <t>INT</t>
         </is>
       </c>
-      <c r="D12" s="11" t="inlineStr">
+      <c r="D12" s="20" t="inlineStr">
         <is>
           <t>PRIMARY KEY, AUTO_INCREMENT</t>
         </is>
       </c>
-      <c r="E12" s="11" t="inlineStr">
+      <c r="E12" s="20" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="F12" s="11" t="inlineStr">
+      <c r="F12" s="20" t="inlineStr">
         <is>
           <t>Unique product serial ID</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="12" t="inlineStr">
+      <c r="A13" s="21" t="inlineStr">
         <is>
           <t>products</t>
         </is>
       </c>
-      <c r="B13" s="12" t="inlineStr">
+      <c r="B13" s="21" t="inlineStr">
         <is>
           <t>category_id</t>
         </is>
       </c>
-      <c r="C13" s="12" t="inlineStr">
+      <c r="C13" s="21" t="inlineStr">
         <is>
           <t>INT</t>
         </is>
       </c>
-      <c r="D13" s="12" t="inlineStr">
+      <c r="D13" s="21" t="inlineStr">
         <is>
           <t>FOREIGN KEY -&gt; categories</t>
         </is>
       </c>
-      <c r="E13" s="12" t="inlineStr">
+      <c r="E13" s="21" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="F13" s="12" t="inlineStr">
+      <c r="F13" s="21" t="inlineStr">
         <is>
           <t>Links product to parent category</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="11" t="inlineStr">
+      <c r="A14" s="20" t="inlineStr">
         <is>
           <t>products</t>
         </is>
       </c>
-      <c r="B14" s="11" t="inlineStr">
+      <c r="B14" s="20" t="inlineStr">
         <is>
           <t>supplier_id</t>
         </is>
       </c>
-      <c r="C14" s="11" t="inlineStr">
+      <c r="C14" s="20" t="inlineStr">
         <is>
           <t>INT</t>
         </is>
       </c>
-      <c r="D14" s="11" t="inlineStr">
+      <c r="D14" s="20" t="inlineStr">
         <is>
           <t>FOREIGN KEY -&gt; suppliers</t>
         </is>
       </c>
-      <c r="E14" s="11" t="inlineStr">
+      <c r="E14" s="20" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="F14" s="11" t="inlineStr">
+      <c r="F14" s="20" t="inlineStr">
         <is>
           <t>Links product to assigned supplier</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="12" t="inlineStr">
+      <c r="A15" s="21" t="inlineStr">
         <is>
           <t>products</t>
         </is>
       </c>
-      <c r="B15" s="12" t="inlineStr">
+      <c r="B15" s="21" t="inlineStr">
         <is>
           <t>sku</t>
         </is>
       </c>
-      <c r="C15" s="12" t="inlineStr">
+      <c r="C15" s="21" t="inlineStr">
         <is>
           <t>VARCHAR(50)</t>
         </is>
       </c>
-      <c r="D15" s="12" t="inlineStr">
+      <c r="D15" s="21" t="inlineStr">
         <is>
           <t>UNIQUE, NOT NULL</t>
         </is>
       </c>
-      <c r="E15" s="12" t="inlineStr">
+      <c r="E15" s="21" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="F15" s="12" t="inlineStr">
+      <c r="F15" s="21" t="inlineStr">
         <is>
           <t>Stock Keeping Unit code (e.g. PEN001)</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="11" t="inlineStr">
+      <c r="A16" s="20" t="inlineStr">
         <is>
           <t>products</t>
         </is>
       </c>
-      <c r="B16" s="11" t="inlineStr">
+      <c r="B16" s="20" t="inlineStr">
         <is>
           <t>barcode</t>
         </is>
       </c>
-      <c r="C16" s="11" t="inlineStr">
+      <c r="C16" s="20" t="inlineStr">
         <is>
           <t>VARCHAR(50)</t>
         </is>
       </c>
-      <c r="D16" s="11" t="inlineStr">
+      <c r="D16" s="20" t="inlineStr">
         <is>
           <t>UNIQUE, NULLABLE</t>
         </is>
       </c>
-      <c r="E16" s="11" t="inlineStr">
+      <c r="E16" s="20" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="F16" s="11" t="inlineStr">
+      <c r="F16" s="20" t="inlineStr">
         <is>
           <t>1D/2D barcode numerical representation</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="12" t="inlineStr">
+      <c r="A17" s="21" t="inlineStr">
         <is>
           <t>products</t>
         </is>
       </c>
-      <c r="B17" s="12" t="inlineStr">
+      <c r="B17" s="21" t="inlineStr">
         <is>
           <t>product_name</t>
         </is>
       </c>
-      <c r="C17" s="12" t="inlineStr">
+      <c r="C17" s="21" t="inlineStr">
         <is>
           <t>VARCHAR(150)</t>
         </is>
       </c>
-      <c r="D17" s="12" t="inlineStr">
+      <c r="D17" s="21" t="inlineStr">
         <is>
           <t>NOT NULL</t>
         </is>
       </c>
-      <c r="E17" s="12" t="inlineStr">
+      <c r="E17" s="21" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="F17" s="12" t="inlineStr">
+      <c r="F17" s="21" t="inlineStr">
         <is>
           <t>Full title of the stationery item</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="11" t="inlineStr">
+      <c r="A18" s="20" t="inlineStr">
         <is>
           <t>products</t>
         </is>
       </c>
-      <c r="B18" s="11" t="inlineStr">
+      <c r="B18" s="20" t="inlineStr">
         <is>
           <t>unit_price</t>
         </is>
       </c>
-      <c r="C18" s="11" t="inlineStr">
+      <c r="C18" s="20" t="inlineStr">
         <is>
           <t>DECIMAL(10,2)</t>
         </is>
       </c>
-      <c r="D18" s="11" t="inlineStr">
+      <c r="D18" s="20" t="inlineStr">
         <is>
           <t>NOT NULL, CHECK (price &gt; 0)</t>
         </is>
       </c>
-      <c r="E18" s="11" t="inlineStr">
+      <c r="E18" s="20" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="F18" s="11" t="inlineStr">
+      <c r="F18" s="20" t="inlineStr">
         <is>
           <t>Retail selling price per item in INR</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="12" t="inlineStr">
+      <c r="A19" s="21" t="inlineStr">
         <is>
           <t>products</t>
         </is>
       </c>
-      <c r="B19" s="12" t="inlineStr">
+      <c r="B19" s="21" t="inlineStr">
         <is>
           <t>quantity</t>
         </is>
       </c>
-      <c r="C19" s="12" t="inlineStr">
+      <c r="C19" s="21" t="inlineStr">
         <is>
           <t>INT</t>
         </is>
       </c>
-      <c r="D19" s="12" t="inlineStr">
+      <c r="D19" s="21" t="inlineStr">
         <is>
           <t>NOT NULL, CHECK (quantity &gt;= 0)</t>
         </is>
       </c>
-      <c r="E19" s="12" t="inlineStr">
+      <c r="E19" s="21" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="F19" s="12" t="inlineStr">
+      <c r="F19" s="21" t="inlineStr">
         <is>
           <t>Current physical on-shelf stock count</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="11" t="inlineStr">
+      <c r="A20" s="20" t="inlineStr">
         <is>
           <t>products</t>
         </is>
       </c>
-      <c r="B20" s="11" t="inlineStr">
+      <c r="B20" s="20" t="inlineStr">
         <is>
           <t>reorder_point</t>
         </is>
       </c>
-      <c r="C20" s="11" t="inlineStr">
+      <c r="C20" s="20" t="inlineStr">
         <is>
           <t>INT</t>
         </is>
       </c>
-      <c r="D20" s="11" t="inlineStr">
+      <c r="D20" s="20" t="inlineStr">
         <is>
           <t>NOT NULL, CHECK (reorder &gt;= 1)</t>
         </is>
       </c>
-      <c r="E20" s="11" t="inlineStr">
+      <c r="E20" s="20" t="inlineStr">
         <is>
           <t>10</t>
         </is>
       </c>
-      <c r="F20" s="11" t="inlineStr">
+      <c r="F20" s="20" t="inlineStr">
         <is>
           <t>Safety threshold triggering reorder warnings</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="12" t="inlineStr">
+      <c r="A21" s="21" t="inlineStr">
         <is>
           <t>products</t>
         </is>
       </c>
-      <c r="B21" s="12" t="inlineStr">
+      <c r="B21" s="21" t="inlineStr">
         <is>
           <t>bin_location</t>
         </is>
       </c>
-      <c r="C21" s="12" t="inlineStr">
+      <c r="C21" s="21" t="inlineStr">
         <is>
           <t>VARCHAR(50)</t>
         </is>
       </c>
-      <c r="D21" s="12" t="inlineStr">
+      <c r="D21" s="21" t="inlineStr">
         <is>
           <t>NULLABLE</t>
         </is>
       </c>
-      <c r="E21" s="12" t="inlineStr">
+      <c r="E21" s="21" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="F21" s="12" t="inlineStr">
+      <c r="F21" s="21" t="inlineStr">
         <is>
           <t>Shelf aisle coordinates (e.g. A01, B02)</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="11" t="inlineStr">
+      <c r="A22" s="20" t="inlineStr">
         <is>
           <t>stock_transactions</t>
         </is>
       </c>
-      <c r="B22" s="11" t="inlineStr">
+      <c r="B22" s="20" t="inlineStr">
         <is>
           <t>transaction_id</t>
         </is>
       </c>
-      <c r="C22" s="11" t="inlineStr">
+      <c r="C22" s="20" t="inlineStr">
         <is>
           <t>INT</t>
         </is>
       </c>
-      <c r="D22" s="11" t="inlineStr">
+      <c r="D22" s="20" t="inlineStr">
         <is>
           <t>PRIMARY KEY, AUTO_INCREMENT</t>
         </is>
       </c>
-      <c r="E22" s="11" t="inlineStr">
+      <c r="E22" s="20" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="F22" s="11" t="inlineStr">
+      <c r="F22" s="20" t="inlineStr">
         <is>
           <t>Audit transaction identifier</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="12" t="inlineStr">
+      <c r="A23" s="21" t="inlineStr">
         <is>
           <t>stock_transactions</t>
         </is>
       </c>
-      <c r="B23" s="12" t="inlineStr">
+      <c r="B23" s="21" t="inlineStr">
         <is>
           <t>product_id</t>
         </is>
       </c>
-      <c r="C23" s="12" t="inlineStr">
+      <c r="C23" s="21" t="inlineStr">
         <is>
           <t>INT</t>
         </is>
       </c>
-      <c r="D23" s="12" t="inlineStr">
+      <c r="D23" s="21" t="inlineStr">
         <is>
           <t>FOREIGN KEY -&gt; products</t>
         </is>
       </c>
-      <c r="E23" s="12" t="inlineStr">
+      <c r="E23" s="21" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="F23" s="12" t="inlineStr">
+      <c r="F23" s="21" t="inlineStr">
         <is>
           <t>Associated product reference</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="11" t="inlineStr">
+      <c r="A24" s="20" t="inlineStr">
         <is>
           <t>stock_transactions</t>
         </is>
       </c>
-      <c r="B24" s="11" t="inlineStr">
+      <c r="B24" s="20" t="inlineStr">
         <is>
           <t>transaction_type</t>
         </is>
       </c>
-      <c r="C24" s="11" t="inlineStr">
+      <c r="C24" s="20" t="inlineStr">
         <is>
           <t>ENUM('INWARD','OUTWARD','DAMAGED')</t>
         </is>
       </c>
-      <c r="D24" s="11" t="inlineStr">
+      <c r="D24" s="20" t="inlineStr">
         <is>
           <t>NOT NULL</t>
         </is>
       </c>
-      <c r="E24" s="11" t="inlineStr">
+      <c r="E24" s="20" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="F24" s="11" t="inlineStr">
+      <c r="F24" s="20" t="inlineStr">
         <is>
           <t>Classification of stock movement</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="12" t="inlineStr">
+      <c r="A25" s="21" t="inlineStr">
         <is>
           <t>stock_transactions</t>
         </is>
       </c>
-      <c r="B25" s="12" t="inlineStr">
+      <c r="B25" s="21" t="inlineStr">
         <is>
           <t>quantity</t>
         </is>
       </c>
-      <c r="C25" s="12" t="inlineStr">
+      <c r="C25" s="21" t="inlineStr">
         <is>
           <t>INT</t>
         </is>
       </c>
-      <c r="D25" s="12" t="inlineStr">
+      <c r="D25" s="21" t="inlineStr">
         <is>
           <t>NOT NULL, CHECK (quantity &gt; 0)</t>
         </is>
       </c>
-      <c r="E25" s="12" t="inlineStr">
+      <c r="E25" s="21" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="F25" s="12" t="inlineStr">
+      <c r="F25" s="21" t="inlineStr">
         <is>
           <t>Number of units adjusted</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="11" t="inlineStr">
+      <c r="A26" s="20" t="inlineStr">
         <is>
           <t>stock_transactions</t>
         </is>
       </c>
-      <c r="B26" s="11" t="inlineStr">
+      <c r="B26" s="20" t="inlineStr">
         <is>
           <t>remarks</t>
         </is>
       </c>
-      <c r="C26" s="11" t="inlineStr">
+      <c r="C26" s="20" t="inlineStr">
         <is>
           <t>VARCHAR(255)</t>
         </is>
       </c>
-      <c r="D26" s="11" t="inlineStr">
+      <c r="D26" s="20" t="inlineStr">
         <is>
           <t>NULLABLE</t>
         </is>
       </c>
-      <c r="E26" s="11" t="inlineStr">
+      <c r="E26" s="20" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="F26" s="11" t="inlineStr">
+      <c r="F26" s="20" t="inlineStr">
         <is>
           <t>Reason or purchase invoice note</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="12" t="inlineStr">
+      <c r="A27" s="21" t="inlineStr">
         <is>
           <t>stock_transactions</t>
         </is>
       </c>
-      <c r="B27" s="12" t="inlineStr">
+      <c r="B27" s="21" t="inlineStr">
         <is>
           <t>transaction_date</t>
         </is>
       </c>
-      <c r="C27" s="12" t="inlineStr">
+      <c r="C27" s="21" t="inlineStr">
         <is>
           <t>TIMESTAMP</t>
         </is>
       </c>
-      <c r="D27" s="12" t="inlineStr">
+      <c r="D27" s="21" t="inlineStr">
         <is>
           <t>NOT NULL</t>
         </is>
       </c>
-      <c r="E27" s="12" t="inlineStr">
+      <c r="E27" s="21" t="inlineStr">
         <is>
           <t>CURRENT_TIMESTAMP</t>
         </is>
       </c>
-      <c r="F27" s="12" t="inlineStr">
+      <c r="F27" s="21" t="inlineStr">
         <is>
           <t>Immutable timestamp of event</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="11" t="inlineStr">
+      <c r="A28" s="20" t="inlineStr">
         <is>
           <t>sales</t>
         </is>
       </c>
-      <c r="B28" s="11" t="inlineStr">
+      <c r="B28" s="20" t="inlineStr">
         <is>
           <t>sale_id</t>
         </is>
       </c>
-      <c r="C28" s="11" t="inlineStr">
+      <c r="C28" s="20" t="inlineStr">
         <is>
           <t>INT</t>
         </is>
       </c>
-      <c r="D28" s="11" t="inlineStr">
+      <c r="D28" s="20" t="inlineStr">
         <is>
           <t>PRIMARY KEY, AUTO_INCREMENT</t>
         </is>
       </c>
-      <c r="E28" s="11" t="inlineStr">
+      <c r="E28" s="20" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="F28" s="11" t="inlineStr">
+      <c r="F28" s="20" t="inlineStr">
         <is>
           <t>Customer receipt sale identifier</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="12" t="inlineStr">
+      <c r="A29" s="21" t="inlineStr">
         <is>
           <t>sales</t>
         </is>
       </c>
-      <c r="B29" s="12" t="inlineStr">
+      <c r="B29" s="21" t="inlineStr">
         <is>
           <t>product_id</t>
         </is>
       </c>
-      <c r="C29" s="12" t="inlineStr">
+      <c r="C29" s="21" t="inlineStr">
         <is>
           <t>INT</t>
         </is>
       </c>
-      <c r="D29" s="12" t="inlineStr">
+      <c r="D29" s="21" t="inlineStr">
         <is>
           <t>FOREIGN KEY -&gt; products</t>
         </is>
       </c>
-      <c r="E29" s="12" t="inlineStr">
+      <c r="E29" s="21" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="F29" s="12" t="inlineStr">
+      <c r="F29" s="21" t="inlineStr">
         <is>
           <t>Product sold reference</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="11" t="inlineStr">
+      <c r="A30" s="20" t="inlineStr">
         <is>
           <t>sales</t>
         </is>
       </c>
-      <c r="B30" s="11" t="inlineStr">
+      <c r="B30" s="20" t="inlineStr">
         <is>
           <t>quantity_sold</t>
         </is>
       </c>
-      <c r="C30" s="11" t="inlineStr">
+      <c r="C30" s="20" t="inlineStr">
         <is>
           <t>INT</t>
         </is>
       </c>
-      <c r="D30" s="11" t="inlineStr">
+      <c r="D30" s="20" t="inlineStr">
         <is>
           <t>NOT NULL, CHECK (quantity &gt; 0)</t>
         </is>
       </c>
-      <c r="E30" s="11" t="inlineStr">
+      <c r="E30" s="20" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="F30" s="11" t="inlineStr">
+      <c r="F30" s="20" t="inlineStr">
         <is>
           <t>Units purchased at counter</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="12" t="inlineStr">
+      <c r="A31" s="21" t="inlineStr">
         <is>
           <t>sales</t>
         </is>
       </c>
-      <c r="B31" s="12" t="inlineStr">
+      <c r="B31" s="21" t="inlineStr">
         <is>
           <t>total_price</t>
         </is>
       </c>
-      <c r="C31" s="12" t="inlineStr">
+      <c r="C31" s="21" t="inlineStr">
         <is>
           <t>DECIMAL(10,2)</t>
         </is>
       </c>
-      <c r="D31" s="12" t="inlineStr">
+      <c r="D31" s="21" t="inlineStr">
         <is>
           <t>NOT NULL</t>
         </is>
       </c>
-      <c r="E31" s="12" t="inlineStr">
+      <c r="E31" s="21" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="F31" s="12" t="inlineStr">
+      <c r="F31" s="21" t="inlineStr">
         <is>
           <t>Calculated bill amount in INR</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="11" t="inlineStr">
+      <c r="A32" s="20" t="inlineStr">
         <is>
           <t>sales</t>
         </is>
       </c>
-      <c r="B32" s="11" t="inlineStr">
+      <c r="B32" s="20" t="inlineStr">
         <is>
           <t>sale_date</t>
         </is>
       </c>
-      <c r="C32" s="11" t="inlineStr">
+      <c r="C32" s="20" t="inlineStr">
         <is>
           <t>TIMESTAMP</t>
         </is>
       </c>
-      <c r="D32" s="11" t="inlineStr">
+      <c r="D32" s="20" t="inlineStr">
         <is>
           <t>NOT NULL</t>
         </is>
       </c>
-      <c r="E32" s="11" t="inlineStr">
+      <c r="E32" s="20" t="inlineStr">
         <is>
           <t>CURRENT_TIMESTAMP</t>
         </is>
       </c>
-      <c r="F32" s="11" t="inlineStr">
+      <c r="F32" s="20" t="inlineStr">
         <is>
           <t>Date and time of customer purchase</t>
         </is>
@@ -2767,12 +3106,12 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:F20"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="39" customWidth="1" min="1" max="1"/>
     <col width="26" customWidth="1" min="2" max="2"/>
-    <col width="48" customWidth="1" min="3" max="3"/>
-    <col width="48" customWidth="1" min="4" max="4"/>
+    <col width="49" customWidth="1" min="3" max="3"/>
+    <col width="55" customWidth="1" min="4" max="4"/>
     <col width="39" customWidth="1" min="5" max="5"/>
     <col width="35" customWidth="1" min="6" max="6"/>
   </cols>
@@ -2785,577 +3124,577 @@
       </c>
     </row>
     <row r="2"/>
-    <row r="3" ht="25" customHeight="1">
-      <c r="A3" s="8" t="inlineStr">
+    <row r="3" ht="26" customHeight="1">
+      <c r="A3" s="15" t="inlineStr">
         <is>
           <t>HTTP Method</t>
         </is>
       </c>
-      <c r="B3" s="8" t="inlineStr">
+      <c r="B3" s="15" t="inlineStr">
         <is>
           <t>Endpoint URL</t>
         </is>
       </c>
-      <c r="C3" s="8" t="inlineStr">
+      <c r="C3" s="15" t="inlineStr">
         <is>
           <t>Purpose &amp; Business Function</t>
         </is>
       </c>
-      <c r="D3" s="8" t="inlineStr">
+      <c r="D3" s="15" t="inlineStr">
         <is>
           <t>Request Payload (JSON)</t>
         </is>
       </c>
-      <c r="E3" s="8" t="inlineStr">
+      <c r="E3" s="15" t="inlineStr">
         <is>
           <t>Success Response</t>
         </is>
       </c>
-      <c r="F3" s="8" t="inlineStr">
+      <c r="F3" s="15" t="inlineStr">
         <is>
           <t>Error Codes</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="9" t="inlineStr">
+      <c r="A4" s="18" t="inlineStr">
         <is>
           <t>GET</t>
         </is>
       </c>
-      <c r="B4" s="9" t="inlineStr">
+      <c r="B4" s="18" t="inlineStr">
         <is>
           <t>/api/products</t>
         </is>
       </c>
-      <c r="C4" s="9" t="inlineStr">
+      <c r="C4" s="18" t="inlineStr">
         <is>
           <t>Fetch all products with live search &amp; filters</t>
         </is>
       </c>
-      <c r="D4" s="9" t="inlineStr">
+      <c r="D4" s="18" t="inlineStr">
         <is>
           <t>Query parameters (?search=, ?category=, ?status=)</t>
         </is>
       </c>
-      <c r="E4" s="9" t="inlineStr">
+      <c r="E4" s="18" t="inlineStr">
         <is>
           <t>200 OK with JSON array of products</t>
         </is>
       </c>
-      <c r="F4" s="9" t="inlineStr">
+      <c r="F4" s="18" t="inlineStr">
         <is>
           <t>500 Server Error</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="10" t="inlineStr">
+      <c r="A5" s="19" t="inlineStr">
         <is>
           <t>POST</t>
         </is>
       </c>
-      <c r="B5" s="10" t="inlineStr">
+      <c r="B5" s="19" t="inlineStr">
         <is>
           <t>/api/products</t>
         </is>
       </c>
-      <c r="C5" s="10" t="inlineStr">
+      <c r="C5" s="19" t="inlineStr">
         <is>
           <t>Create new stationery product with validation</t>
         </is>
       </c>
-      <c r="D5" s="10" t="inlineStr">
+      <c r="D5" s="19" t="inlineStr">
         <is>
           <t>{"productName": "...", "sku": "...", "unitPrice": 10, ...}</t>
         </is>
       </c>
-      <c r="E5" s="10" t="inlineStr">
+      <c r="E5" s="19" t="inlineStr">
         <is>
           <t>201 Created with saved product JSON</t>
         </is>
       </c>
-      <c r="F5" s="10" t="inlineStr">
+      <c r="F5" s="19" t="inlineStr">
         <is>
           <t>400 Bad Request / 409 Conflict</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="9" t="inlineStr">
+      <c r="A6" s="18" t="inlineStr">
         <is>
           <t>PUT</t>
         </is>
       </c>
-      <c r="B6" s="9" t="inlineStr">
+      <c r="B6" s="18" t="inlineStr">
         <is>
           <t>/api/products/{id}</t>
         </is>
       </c>
-      <c r="C6" s="9" t="inlineStr">
+      <c r="C6" s="18" t="inlineStr">
         <is>
           <t>Update existing stationery product details</t>
         </is>
       </c>
-      <c r="D6" s="9" t="inlineStr">
+      <c r="D6" s="18" t="inlineStr">
         <is>
           <t>{"productName": "...", "unitPrice": 12, ...}</t>
         </is>
       </c>
-      <c r="E6" s="9" t="inlineStr">
+      <c r="E6" s="18" t="inlineStr">
         <is>
           <t>200 OK with updated product JSON</t>
         </is>
       </c>
-      <c r="F6" s="9" t="inlineStr">
+      <c r="F6" s="18" t="inlineStr">
         <is>
           <t>400 Bad Request / 404 Not Found</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="10" t="inlineStr">
+      <c r="A7" s="19" t="inlineStr">
         <is>
           <t>DELETE</t>
         </is>
       </c>
-      <c r="B7" s="10" t="inlineStr">
+      <c r="B7" s="19" t="inlineStr">
         <is>
           <t>/api/products/{id}</t>
         </is>
       </c>
-      <c r="C7" s="10" t="inlineStr">
+      <c r="C7" s="19" t="inlineStr">
         <is>
           <t>Delete stationery product</t>
         </is>
       </c>
-      <c r="D7" s="10" t="inlineStr">
+      <c r="D7" s="19" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="E7" s="10" t="inlineStr">
+      <c r="E7" s="19" t="inlineStr">
         <is>
           <t>200 OK with {"success": true}</t>
         </is>
       </c>
-      <c r="F7" s="10" t="inlineStr">
+      <c r="F7" s="19" t="inlineStr">
         <is>
           <t>409 Conflict if sales exist</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="9" t="inlineStr">
+      <c r="A8" s="18" t="inlineStr">
         <is>
           <t>GET</t>
         </is>
       </c>
-      <c r="B8" s="9" t="inlineStr">
+      <c r="B8" s="18" t="inlineStr">
         <is>
           <t>/api/categories</t>
         </is>
       </c>
-      <c r="C8" s="9" t="inlineStr">
+      <c r="C8" s="18" t="inlineStr">
         <is>
           <t>List all master categories</t>
         </is>
       </c>
-      <c r="D8" s="9" t="inlineStr">
+      <c r="D8" s="18" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="E8" s="9" t="inlineStr">
+      <c r="E8" s="18" t="inlineStr">
         <is>
           <t>200 OK with categories array</t>
         </is>
       </c>
-      <c r="F8" s="9" t="inlineStr">
+      <c r="F8" s="18" t="inlineStr">
         <is>
           <t>500 Server Error</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="10" t="inlineStr">
+      <c r="A9" s="19" t="inlineStr">
         <is>
           <t>POST</t>
         </is>
       </c>
-      <c r="B9" s="10" t="inlineStr">
+      <c r="B9" s="19" t="inlineStr">
         <is>
           <t>/api/categories</t>
         </is>
       </c>
-      <c r="C9" s="10" t="inlineStr">
+      <c r="C9" s="19" t="inlineStr">
         <is>
           <t>Add new stationery category</t>
         </is>
       </c>
-      <c r="D9" s="10" t="inlineStr">
+      <c r="D9" s="19" t="inlineStr">
         <is>
           <t>{"categoryName": "Pens &amp; Writing"}</t>
         </is>
       </c>
-      <c r="E9" s="10" t="inlineStr">
+      <c r="E9" s="19" t="inlineStr">
         <is>
           <t>201 Created with category JSON</t>
         </is>
       </c>
-      <c r="F9" s="10" t="inlineStr">
+      <c r="F9" s="19" t="inlineStr">
         <is>
           <t>400 Bad Request</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="9" t="inlineStr">
+      <c r="A10" s="18" t="inlineStr">
         <is>
           <t>GET</t>
         </is>
       </c>
-      <c r="B10" s="9" t="inlineStr">
+      <c r="B10" s="18" t="inlineStr">
         <is>
           <t>/api/suppliers</t>
         </is>
       </c>
-      <c r="C10" s="9" t="inlineStr">
+      <c r="C10" s="18" t="inlineStr">
         <is>
           <t>List all vendor suppliers</t>
         </is>
       </c>
-      <c r="D10" s="9" t="inlineStr">
+      <c r="D10" s="18" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="E10" s="9" t="inlineStr">
+      <c r="E10" s="18" t="inlineStr">
         <is>
           <t>200 OK with suppliers array</t>
         </is>
       </c>
-      <c r="F10" s="9" t="inlineStr">
+      <c r="F10" s="18" t="inlineStr">
         <is>
           <t>500 Server Error</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="10" t="inlineStr">
+      <c r="A11" s="19" t="inlineStr">
         <is>
           <t>POST</t>
         </is>
       </c>
-      <c r="B11" s="10" t="inlineStr">
+      <c r="B11" s="19" t="inlineStr">
         <is>
           <t>/api/suppliers</t>
         </is>
       </c>
-      <c r="C11" s="10" t="inlineStr">
+      <c r="C11" s="19" t="inlineStr">
         <is>
           <t>Register new vendor supplier</t>
         </is>
       </c>
-      <c r="D11" s="10" t="inlineStr">
+      <c r="D11" s="19" t="inlineStr">
         <is>
           <t>{"supplierName": "Camlin", "phone": "..."}</t>
         </is>
       </c>
-      <c r="E11" s="10" t="inlineStr">
+      <c r="E11" s="19" t="inlineStr">
         <is>
           <t>201 Created with supplier JSON</t>
         </is>
       </c>
-      <c r="F11" s="10" t="inlineStr">
+      <c r="F11" s="19" t="inlineStr">
         <is>
           <t>400 Bad Request</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="9" t="inlineStr">
+      <c r="A12" s="18" t="inlineStr">
         <is>
           <t>POST</t>
         </is>
       </c>
-      <c r="B12" s="9" t="inlineStr">
+      <c r="B12" s="18" t="inlineStr">
         <is>
           <t>/api/stock/inward</t>
         </is>
       </c>
-      <c r="C12" s="9" t="inlineStr">
+      <c r="C12" s="18" t="inlineStr">
         <is>
           <t>Receive supplier shipment delivery</t>
         </is>
       </c>
-      <c r="D12" s="9" t="inlineStr">
+      <c r="D12" s="18" t="inlineStr">
         <is>
           <t>{"productId": 1, "quantity": 50, "remarks": "..."}</t>
         </is>
       </c>
-      <c r="E12" s="9" t="inlineStr">
+      <c r="E12" s="18" t="inlineStr">
         <is>
           <t>200 OK with transaction JSON</t>
         </is>
       </c>
-      <c r="F12" s="9" t="inlineStr">
+      <c r="F12" s="18" t="inlineStr">
         <is>
           <t>400 Bad Request</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="10" t="inlineStr">
+      <c r="A13" s="19" t="inlineStr">
         <is>
           <t>POST</t>
         </is>
       </c>
-      <c r="B13" s="10" t="inlineStr">
+      <c r="B13" s="19" t="inlineStr">
         <is>
           <t>/api/stock/outward</t>
         </is>
       </c>
-      <c r="C13" s="10" t="inlineStr">
+      <c r="C13" s="19" t="inlineStr">
         <is>
           <t>Record internal dispatch / bulk issue</t>
         </is>
       </c>
-      <c r="D13" s="10" t="inlineStr">
+      <c r="D13" s="19" t="inlineStr">
         <is>
           <t>{"productId": 1, "quantity": 10, "remarks": "..."}</t>
         </is>
       </c>
-      <c r="E13" s="10" t="inlineStr">
+      <c r="E13" s="19" t="inlineStr">
         <is>
           <t>200 OK with transaction JSON</t>
         </is>
       </c>
-      <c r="F13" s="10" t="inlineStr">
+      <c r="F13" s="19" t="inlineStr">
         <is>
           <t>400 Insufficient Stock</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="9" t="inlineStr">
+      <c r="A14" s="18" t="inlineStr">
         <is>
           <t>POST</t>
         </is>
       </c>
-      <c r="B14" s="9" t="inlineStr">
+      <c r="B14" s="18" t="inlineStr">
         <is>
           <t>/api/stock/damaged</t>
         </is>
       </c>
-      <c r="C14" s="9" t="inlineStr">
+      <c r="C14" s="18" t="inlineStr">
         <is>
           <t>Write off broken / dried-up stationery</t>
         </is>
       </c>
-      <c r="D14" s="9" t="inlineStr">
+      <c r="D14" s="18" t="inlineStr">
         <is>
           <t>{"productId": 1, "quantity": 2, "remarks": "..."}</t>
         </is>
       </c>
-      <c r="E14" s="9" t="inlineStr">
+      <c r="E14" s="18" t="inlineStr">
         <is>
           <t>200 OK with transaction JSON</t>
         </is>
       </c>
-      <c r="F14" s="9" t="inlineStr">
+      <c r="F14" s="18" t="inlineStr">
         <is>
           <t>400 Insufficient Stock</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="10" t="inlineStr">
+      <c r="A15" s="19" t="inlineStr">
         <is>
           <t>GET</t>
         </is>
       </c>
-      <c r="B15" s="10" t="inlineStr">
+      <c r="B15" s="19" t="inlineStr">
         <is>
           <t>/api/stock/history</t>
         </is>
       </c>
-      <c r="C15" s="10" t="inlineStr">
+      <c r="C15" s="19" t="inlineStr">
         <is>
           <t>Retrieve immutable audit ledger records</t>
         </is>
       </c>
-      <c r="D15" s="10" t="inlineStr">
+      <c r="D15" s="19" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="E15" s="10" t="inlineStr">
+      <c r="E15" s="19" t="inlineStr">
         <is>
           <t>200 OK with transaction array</t>
         </is>
       </c>
-      <c r="F15" s="10" t="inlineStr">
+      <c r="F15" s="19" t="inlineStr">
         <is>
           <t>500 Server Error</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="9" t="inlineStr">
+      <c r="A16" s="18" t="inlineStr">
         <is>
           <t>POST</t>
         </is>
       </c>
-      <c r="B16" s="9" t="inlineStr">
+      <c r="B16" s="18" t="inlineStr">
         <is>
           <t>/api/sales</t>
         </is>
       </c>
-      <c r="C16" s="9" t="inlineStr">
+      <c r="C16" s="18" t="inlineStr">
         <is>
           <t>Execute atomic POS customer checkout</t>
         </is>
       </c>
-      <c r="D16" s="9" t="inlineStr">
+      <c r="D16" s="18" t="inlineStr">
         <is>
           <t>{"productId": 1, "quantitySold": 5}</t>
         </is>
       </c>
-      <c r="E16" s="9" t="inlineStr">
+      <c r="E16" s="18" t="inlineStr">
         <is>
           <t>201 Created with sale JSON</t>
         </is>
       </c>
-      <c r="F16" s="9" t="inlineStr">
+      <c r="F16" s="18" t="inlineStr">
         <is>
           <t>400 Out of Stock</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="10" t="inlineStr">
+      <c r="A17" s="19" t="inlineStr">
         <is>
           <t>GET</t>
         </is>
       </c>
-      <c r="B17" s="10" t="inlineStr">
+      <c r="B17" s="19" t="inlineStr">
         <is>
           <t>/api/sales</t>
         </is>
       </c>
-      <c r="C17" s="10" t="inlineStr">
+      <c r="C17" s="19" t="inlineStr">
         <is>
           <t>Fetch recent customer sales register</t>
         </is>
       </c>
-      <c r="D17" s="10" t="inlineStr">
+      <c r="D17" s="19" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="E17" s="10" t="inlineStr">
+      <c r="E17" s="19" t="inlineStr">
         <is>
           <t>200 OK with sales array</t>
         </is>
       </c>
-      <c r="F17" s="10" t="inlineStr">
+      <c r="F17" s="19" t="inlineStr">
         <is>
           <t>500 Server Error</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="9" t="inlineStr">
+      <c r="A18" s="18" t="inlineStr">
         <is>
           <t>GET</t>
         </is>
       </c>
-      <c r="B18" s="9" t="inlineStr">
+      <c r="B18" s="18" t="inlineStr">
         <is>
           <t>/api/reports/dashboard</t>
         </is>
       </c>
-      <c r="C18" s="9" t="inlineStr">
+      <c r="C18" s="18" t="inlineStr">
         <is>
           <t>Compute 4 live store KPI metrics</t>
         </is>
       </c>
-      <c r="D18" s="9" t="inlineStr">
+      <c r="D18" s="18" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="E18" s="9" t="inlineStr">
+      <c r="E18" s="18" t="inlineStr">
         <is>
           <t>200 OK with KPI summary JSON</t>
         </is>
       </c>
-      <c r="F18" s="9" t="inlineStr">
+      <c r="F18" s="18" t="inlineStr">
         <is>
           <t>500 Server Error</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="10" t="inlineStr">
+      <c r="A19" s="19" t="inlineStr">
         <is>
           <t>GET</t>
         </is>
       </c>
-      <c r="B19" s="10" t="inlineStr">
+      <c r="B19" s="19" t="inlineStr">
         <is>
           <t>/api/reports/low-stock</t>
         </is>
       </c>
-      <c r="C19" s="10" t="inlineStr">
+      <c r="C19" s="19" t="inlineStr">
         <is>
           <t>Filter items at or below reorder point</t>
         </is>
       </c>
-      <c r="D19" s="10" t="inlineStr">
+      <c r="D19" s="19" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="E19" s="10" t="inlineStr">
+      <c r="E19" s="19" t="inlineStr">
         <is>
           <t>200 OK with low-stock array</t>
         </is>
       </c>
-      <c r="F19" s="10" t="inlineStr">
+      <c r="F19" s="19" t="inlineStr">
         <is>
           <t>500 Server Error</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="9" t="inlineStr">
+      <c r="A20" s="18" t="inlineStr">
         <is>
           <t>GET</t>
         </is>
       </c>
-      <c r="B20" s="9" t="inlineStr">
+      <c r="B20" s="18" t="inlineStr">
         <is>
           <t>/api/reports/valuation</t>
         </is>
       </c>
-      <c r="C20" s="9" t="inlineStr">
+      <c r="C20" s="18" t="inlineStr">
         <is>
           <t>Aggregate financial valuation by category</t>
         </is>
       </c>
-      <c r="D20" s="9" t="inlineStr">
+      <c r="D20" s="18" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="E20" s="9" t="inlineStr">
+      <c r="E20" s="18" t="inlineStr">
         <is>
           <t>200 OK with valuation array</t>
         </is>
       </c>
-      <c r="F20" s="9" t="inlineStr">
+      <c r="F20" s="18" t="inlineStr">
         <is>
           <t>500 Server Error</t>
         </is>
@@ -3373,13 +3712,13 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:E7"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
-    <col width="48" customWidth="1" min="1" max="1"/>
+    <col width="51" customWidth="1" min="1" max="1"/>
     <col width="27" customWidth="1" min="2" max="2"/>
     <col width="34" customWidth="1" min="3" max="3"/>
-    <col width="48" customWidth="1" min="4" max="4"/>
-    <col width="48" customWidth="1" min="5" max="5"/>
+    <col width="55" customWidth="1" min="4" max="4"/>
+    <col width="55" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3390,136 +3729,136 @@
       </c>
     </row>
     <row r="2"/>
-    <row r="3" ht="25" customHeight="1">
-      <c r="A3" s="8" t="inlineStr">
+    <row r="3" ht="26" customHeight="1">
+      <c r="A3" s="15" t="inlineStr">
         <is>
           <t>SDLC Phase</t>
         </is>
       </c>
-      <c r="B3" s="8" t="inlineStr">
+      <c r="B3" s="15" t="inlineStr">
         <is>
           <t>CARE Element</t>
         </is>
       </c>
-      <c r="C3" s="8" t="inlineStr">
+      <c r="C3" s="15" t="inlineStr">
         <is>
           <t>Prompt Objective / Action</t>
         </is>
       </c>
-      <c r="D3" s="8" t="inlineStr">
+      <c r="D3" s="15" t="inlineStr">
         <is>
           <t>Input Prompt Details</t>
         </is>
       </c>
-      <c r="E3" s="8" t="inlineStr">
+      <c r="E3" s="15" t="inlineStr">
         <is>
           <t>Generated Artifact / Verification Result</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="9" t="inlineStr">
+      <c r="A4" s="18" t="inlineStr">
         <is>
           <t>Phase 1: DEFINE</t>
         </is>
       </c>
-      <c r="B4" s="9" t="inlineStr">
+      <c r="B4" s="18" t="inlineStr">
         <is>
           <t>Context &amp; Action</t>
         </is>
       </c>
-      <c r="C4" s="9" t="inlineStr">
+      <c r="C4" s="18" t="inlineStr">
         <is>
           <t>Requirements Specification</t>
         </is>
       </c>
-      <c r="D4" s="9" t="inlineStr">
+      <c r="D4" s="18" t="inlineStr">
         <is>
           <t>Define scope, personas, user stories, and acceptance criteria for Smart Stationery Inventory System.</t>
         </is>
       </c>
-      <c r="E4" s="9" t="inlineStr">
+      <c r="E4" s="18" t="inlineStr">
         <is>
           <t>Created docs/DEFINE.md with 6 user stories and Given/When/Then criteria.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="10" t="inlineStr">
+      <c r="A5" s="19" t="inlineStr">
         <is>
           <t>Phase 2: DESIGN</t>
         </is>
       </c>
-      <c r="B5" s="10" t="inlineStr">
+      <c r="B5" s="19" t="inlineStr">
         <is>
           <t>Action &amp; Result</t>
         </is>
       </c>
-      <c r="C5" s="10" t="inlineStr">
+      <c r="C5" s="19" t="inlineStr">
         <is>
           <t>Architecture &amp; Schema Design</t>
         </is>
       </c>
-      <c r="D5" s="10" t="inlineStr">
+      <c r="D5" s="19" t="inlineStr">
         <is>
           <t>Design 3-tier architecture, DFD level 0 &amp; 1, and 3NF MySQL schema with non-negative constraints.</t>
         </is>
       </c>
-      <c r="E5" s="10" t="inlineStr">
+      <c r="E5" s="19" t="inlineStr">
         <is>
           <t>Generated docs/DESIGN.md, docs/architecture.md, database/schema.sql and sample_data.sql.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="9" t="inlineStr">
+      <c r="A6" s="18" t="inlineStr">
         <is>
           <t>Phase 3: DEVELOP</t>
         </is>
       </c>
-      <c r="B6" s="9" t="inlineStr">
+      <c r="B6" s="18" t="inlineStr">
         <is>
           <t>Action &amp; Result</t>
         </is>
       </c>
-      <c r="C6" s="9" t="inlineStr">
-        <is>
-          <t>Pure Java SE &amp; Vanilla Web</t>
-        </is>
-      </c>
-      <c r="D6" s="9" t="inlineStr">
-        <is>
-          <t>Implement SimpleHttpServer with Virtual Threads, plain JDBC PreparedStatement, and Vanilla HTML/CSS/JS frontend.</t>
-        </is>
-      </c>
-      <c r="E6" s="9" t="inlineStr">
-        <is>
-          <t>Produced backend/src/ classes and frontend/ (index.html, style.css, script.js). 100% test pass.</t>
+      <c r="C6" s="18" t="inlineStr">
+        <is>
+          <t>Core Java SE &amp; React FullStack</t>
+        </is>
+      </c>
+      <c r="D6" s="18" t="inlineStr">
+        <is>
+          <t>Implement SimpleHttpServer with Virtual Threads, plain JDBC PreparedStatement, React 19 UI &amp; Vanilla Web.</t>
+        </is>
+      </c>
+      <c r="E6" s="18" t="inlineStr">
+        <is>
+          <t>Produced backend/src/ classes, frontend/ React components, and static web. 100% test pass.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="10" t="inlineStr">
+      <c r="A7" s="19" t="inlineStr">
         <is>
           <t>Phase 4: DEPLOY</t>
         </is>
       </c>
-      <c r="B7" s="10" t="inlineStr">
+      <c r="B7" s="19" t="inlineStr">
         <is>
           <t>Examples &amp; Verification</t>
         </is>
       </c>
-      <c r="C7" s="10" t="inlineStr">
+      <c r="C7" s="19" t="inlineStr">
         <is>
           <t>Runbook, Presentation &amp; Runner</t>
         </is>
       </c>
-      <c r="D7" s="10" t="inlineStr">
-        <is>
-          <t>Generate 12-sheet Excel runbook, 20-slide projector presentation, and 1-click run.bat startup script.</t>
-        </is>
-      </c>
-      <c r="E7" s="10" t="inlineStr">
+      <c r="D7" s="19" t="inlineStr">
+        <is>
+          <t>Generate SIST 12-sheet Excel runbook, 20-slide projector presentation, and 1-click run.bat startup script.</t>
+        </is>
+      </c>
+      <c r="E7" s="19" t="inlineStr">
         <is>
           <t>Generated docs/Student_FullStack_Project_Runbook.xlsx, presentation/presentation.html, and run.bat.</t>
         </is>
@@ -3537,236 +3876,236 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:E10"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
-    <col width="48" customWidth="1" min="1" max="1"/>
-    <col width="23" customWidth="1" min="2" max="2"/>
-    <col width="34" customWidth="1" min="3" max="3"/>
-    <col width="48" customWidth="1" min="4" max="4"/>
-    <col width="48" customWidth="1" min="5" max="5"/>
+    <col width="55" customWidth="1" min="1" max="1"/>
+    <col width="38" customWidth="1" min="2" max="2"/>
+    <col width="35" customWidth="1" min="3" max="3"/>
+    <col width="50" customWidth="1" min="4" max="4"/>
+    <col width="55" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>FRONTEND UI COMPONENT SPECIFICATIONS (HTML5 / CSS3)</t>
+          <t>FRONTEND UI COMPONENT SPECIFICATIONS (REACT 19 &amp; HTML5/CSS3)</t>
         </is>
       </c>
     </row>
     <row r="2"/>
-    <row r="3" ht="25" customHeight="1">
-      <c r="A3" s="8" t="inlineStr">
+    <row r="3" ht="26" customHeight="1">
+      <c r="A3" s="15" t="inlineStr">
         <is>
           <t>Component ID</t>
         </is>
       </c>
-      <c r="B3" s="8" t="inlineStr">
+      <c r="B3" s="15" t="inlineStr">
         <is>
           <t>File Location</t>
         </is>
       </c>
-      <c r="C3" s="8" t="inlineStr">
+      <c r="C3" s="15" t="inlineStr">
         <is>
           <t>Element Type</t>
         </is>
       </c>
-      <c r="D3" s="8" t="inlineStr">
+      <c r="D3" s="15" t="inlineStr">
         <is>
           <t>CSS Styling Technique</t>
         </is>
       </c>
-      <c r="E3" s="8" t="inlineStr">
+      <c r="E3" s="15" t="inlineStr">
         <is>
           <t>Functional Behavior &amp; Interaction</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="9" t="inlineStr">
+      <c r="A4" s="18" t="inlineStr">
         <is>
           <t>UI-01</t>
         </is>
       </c>
-      <c r="B4" s="9" t="inlineStr">
-        <is>
-          <t>frontend/index.html</t>
-        </is>
-      </c>
-      <c r="C4" s="9" t="inlineStr">
-        <is>
-          <t>&lt;header class='app-header'&gt;</t>
-        </is>
-      </c>
-      <c r="D4" s="9" t="inlineStr">
+      <c r="B4" s="18" t="inlineStr">
+        <is>
+          <t>frontend/src/pages/Login.jsx</t>
+        </is>
+      </c>
+      <c r="C4" s="18" t="inlineStr">
+        <is>
+          <t>&lt;div className='login-box'&gt;</t>
+        </is>
+      </c>
+      <c r="D4" s="18" t="inlineStr">
+        <is>
+          <t>Glassmorphism card, gradient accent, shadow-xl</t>
+        </is>
+      </c>
+      <c r="E4" s="18" t="inlineStr">
+        <is>
+          <t>Provides secure role-based login for admin, staff1, and staff2 with clear error feedback.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="19" t="inlineStr">
+        <is>
+          <t>UI-02</t>
+        </is>
+      </c>
+      <c r="B5" s="19" t="inlineStr">
+        <is>
+          <t>frontend/src/components/Navbar.jsx</t>
+        </is>
+      </c>
+      <c r="C5" s="19" t="inlineStr">
+        <is>
+          <t>&lt;header className='app-header'&gt;</t>
+        </is>
+      </c>
+      <c r="D5" s="19" t="inlineStr">
         <is>
           <t>Flexbox, shadow-sm, academic branding</t>
         </is>
       </c>
-      <c r="E4" s="9" t="inlineStr">
-        <is>
-          <t>Displays system title, live server status indicator (:8080), and student register numbers.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="10" t="inlineStr">
-        <is>
-          <t>UI-02</t>
-        </is>
-      </c>
-      <c r="B5" s="10" t="inlineStr">
-        <is>
-          <t>frontend/index.html</t>
-        </is>
-      </c>
-      <c r="C5" s="10" t="inlineStr">
-        <is>
-          <t>&lt;nav class='app-nav'&gt;</t>
-        </is>
-      </c>
-      <c r="D5" s="10" t="inlineStr">
-        <is>
-          <t>Sticky navigation bar, border-bottom</t>
-        </is>
-      </c>
-      <c r="E5" s="10" t="inlineStr">
-        <is>
-          <t>Houses 7 tab buttons (Dashboard, Products, Categories, Suppliers, Stock, Sales, Reports).</t>
+      <c r="E5" s="19" t="inlineStr">
+        <is>
+          <t>Displays system title, user role badge (Admin/Staff), live server status, and logout action.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="9" t="inlineStr">
+      <c r="A6" s="18" t="inlineStr">
         <is>
           <t>UI-03</t>
         </is>
       </c>
-      <c r="B6" s="9" t="inlineStr">
-        <is>
-          <t>frontend/index.html</t>
-        </is>
-      </c>
-      <c r="C6" s="9" t="inlineStr">
+      <c r="B6" s="18" t="inlineStr">
+        <is>
+          <t>frontend/src/pages/Dashboard.jsx</t>
+        </is>
+      </c>
+      <c r="C6" s="18" t="inlineStr">
         <is>
           <t>.kpi-grid &amp; .kpi-card</t>
         </is>
       </c>
-      <c r="D6" s="9" t="inlineStr">
+      <c r="D6" s="18" t="inlineStr">
         <is>
           <t>CSS Grid (repeat auto-fit minmax 240px)</t>
         </is>
       </c>
-      <c r="E6" s="9" t="inlineStr">
-        <is>
-          <t>Renders 4 metric summary cards with color-coded accent icons (Blue, Green, Amber, Purple).</t>
+      <c r="E6" s="18" t="inlineStr">
+        <is>
+          <t>Renders 4 metric summary cards with color-coded accent icons (Total SKUs, Valuation, Low Stock, Sales).</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="10" t="inlineStr">
+      <c r="A7" s="19" t="inlineStr">
         <is>
           <t>UI-04</t>
         </is>
       </c>
-      <c r="B7" s="10" t="inlineStr">
-        <is>
-          <t>frontend/index.html</t>
-        </is>
-      </c>
-      <c r="C7" s="10" t="inlineStr">
-        <is>
-          <t>.data-table</t>
-        </is>
-      </c>
-      <c r="D7" s="10" t="inlineStr">
-        <is>
-          <t>Border-collapse, light slate hover rows</t>
-        </is>
-      </c>
-      <c r="E7" s="10" t="inlineStr">
-        <is>
-          <t>Presents real-time relational tables for products, low-stock alerts, stock audit, and sales.</t>
+      <c r="B7" s="19" t="inlineStr">
+        <is>
+          <t>frontend/src/pages/Products.jsx</t>
+        </is>
+      </c>
+      <c r="C7" s="19" t="inlineStr">
+        <is>
+          <t>.data-table &amp; search/filter bar</t>
+        </is>
+      </c>
+      <c r="D7" s="19" t="inlineStr">
+        <is>
+          <t>Border-collapse, hover rows, status badges</t>
+        </is>
+      </c>
+      <c r="E7" s="19" t="inlineStr">
+        <is>
+          <t>Presents real-time relational table for products with search, category filtering, and stock badges.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="9" t="inlineStr">
+      <c r="A8" s="18" t="inlineStr">
         <is>
           <t>UI-05</t>
         </is>
       </c>
-      <c r="B8" s="9" t="inlineStr">
-        <is>
-          <t>frontend/index.html</t>
-        </is>
-      </c>
-      <c r="C8" s="9" t="inlineStr">
-        <is>
-          <t>.modal-overlay &amp; .modal-dialog</t>
-        </is>
-      </c>
-      <c r="D8" s="9" t="inlineStr">
-        <is>
-          <t>Fixed overlay with blur, pop-in animation</t>
-        </is>
-      </c>
-      <c r="E8" s="9" t="inlineStr">
-        <is>
-          <t>Accessible modal forms for adding/editing products, categories, suppliers, and stock intake.</t>
+      <c r="B8" s="18" t="inlineStr">
+        <is>
+          <t>frontend/src/pages/POS.jsx</t>
+        </is>
+      </c>
+      <c r="C8" s="18" t="inlineStr">
+        <is>
+          <t>.pos-layout &amp; cart register</t>
+        </is>
+      </c>
+      <c r="D8" s="18" t="inlineStr">
+        <is>
+          <t>Responsive 2-column POS layout (Form + Cart)</t>
+        </is>
+      </c>
+      <c r="E8" s="18" t="inlineStr">
+        <is>
+          <t>Interactive POS billing screen with instant subtotal updates, overselling guard, and receipt printer.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="10" t="inlineStr">
+      <c r="A9" s="19" t="inlineStr">
         <is>
           <t>UI-06</t>
         </is>
       </c>
-      <c r="B9" s="10" t="inlineStr">
-        <is>
-          <t>frontend/index.html</t>
-        </is>
-      </c>
-      <c r="C9" s="10" t="inlineStr">
-        <is>
-          <t>.pos-layout</t>
-        </is>
-      </c>
-      <c r="D9" s="10" t="inlineStr">
-        <is>
-          <t>Responsive CSS Grid (380px form + 1fr table)</t>
-        </is>
-      </c>
-      <c r="E9" s="10" t="inlineStr">
-        <is>
-          <t>Interactive POS billing screen with instant subtotal updates and receipt register.</t>
+      <c r="B9" s="19" t="inlineStr">
+        <is>
+          <t>frontend/src/pages/Stock.jsx</t>
+        </is>
+      </c>
+      <c r="C9" s="19" t="inlineStr">
+        <is>
+          <t>.modal-overlay &amp; stock ledger</t>
+        </is>
+      </c>
+      <c r="D9" s="19" t="inlineStr">
+        <is>
+          <t>Fixed overlay with backdrop-filter blur</t>
+        </is>
+      </c>
+      <c r="E9" s="19" t="inlineStr">
+        <is>
+          <t>Enables recording inward supplier shipments, outward dispatches, and damaged write-offs.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="9" t="inlineStr">
+      <c r="A10" s="18" t="inlineStr">
         <is>
           <t>UI-07</t>
         </is>
       </c>
-      <c r="B10" s="9" t="inlineStr">
-        <is>
-          <t>frontend/index.html</t>
-        </is>
-      </c>
-      <c r="C10" s="9" t="inlineStr">
-        <is>
-          <t>.toast-container</t>
-        </is>
-      </c>
-      <c r="D10" s="9" t="inlineStr">
-        <is>
-          <t>Fixed bottom-right notification stack</t>
-        </is>
-      </c>
-      <c r="E10" s="9" t="inlineStr">
-        <is>
-          <t>Displays auto-dismissing success and error toast banners after every user action.</t>
+      <c r="B10" s="18" t="inlineStr">
+        <is>
+          <t>frontend/src/pages/Reports.jsx</t>
+        </is>
+      </c>
+      <c r="C10" s="18" t="inlineStr">
+        <is>
+          <t>.report-cards &amp; CSV export</t>
+        </is>
+      </c>
+      <c r="D10" s="18" t="inlineStr">
+        <is>
+          <t>Clean printable grid with CSV download trigger</t>
+        </is>
+      </c>
+      <c r="E10" s="18" t="inlineStr">
+        <is>
+          <t>Generates category valuation summaries, reorder forecasts, and 1-click spreadsheet export.</t>
         </is>
       </c>
     </row>
@@ -3782,13 +4121,13 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:E11"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
-    <col width="48" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="52" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
     <col width="27" customWidth="1" min="3" max="3"/>
     <col width="47" customWidth="1" min="4" max="4"/>
-    <col width="48" customWidth="1" min="5" max="5"/>
+    <col width="55" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3799,244 +4138,244 @@
       </c>
     </row>
     <row r="2"/>
-    <row r="3" ht="25" customHeight="1">
-      <c r="A3" s="8" t="inlineStr">
+    <row r="3" ht="26" customHeight="1">
+      <c r="A3" s="15" t="inlineStr">
         <is>
           <t>Class Name</t>
         </is>
       </c>
-      <c r="B3" s="8" t="inlineStr">
+      <c r="B3" s="15" t="inlineStr">
         <is>
           <t>Package</t>
         </is>
       </c>
-      <c r="C3" s="8" t="inlineStr">
+      <c r="C3" s="15" t="inlineStr">
         <is>
           <t>Pattern / Role</t>
         </is>
       </c>
-      <c r="D3" s="8" t="inlineStr">
+      <c r="D3" s="15" t="inlineStr">
         <is>
           <t>Key Methods</t>
         </is>
       </c>
-      <c r="E3" s="8" t="inlineStr">
+      <c r="E3" s="15" t="inlineStr">
         <is>
           <t>Technical Details &amp; ACID Compliance</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="9" t="inlineStr">
+      <c r="A4" s="18" t="inlineStr">
         <is>
           <t>Main.java</t>
         </is>
       </c>
-      <c r="B4" s="9" t="inlineStr">
+      <c r="B4" s="18" t="inlineStr">
         <is>
           <t>default</t>
         </is>
       </c>
-      <c r="C4" s="9" t="inlineStr">
+      <c r="C4" s="18" t="inlineStr">
         <is>
           <t>Application Entrypoint</t>
         </is>
       </c>
-      <c r="D4" s="9" t="inlineStr">
+      <c r="D4" s="18" t="inlineStr">
         <is>
           <t>main(String[] args)</t>
         </is>
       </c>
-      <c r="E4" s="9" t="inlineStr">
+      <c r="E4" s="18" t="inlineStr">
         <is>
           <t>Initializes database connectivity, runs table verification, and boots SimpleHttpServer on port 8080.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="10" t="inlineStr">
+      <c r="A5" s="19" t="inlineStr">
         <is>
           <t>SimpleHttpServer.java</t>
         </is>
       </c>
-      <c r="B5" s="10" t="inlineStr">
+      <c r="B5" s="19" t="inlineStr">
         <is>
           <t>server</t>
         </is>
       </c>
-      <c r="C5" s="10" t="inlineStr">
+      <c r="C5" s="19" t="inlineStr">
         <is>
           <t>HTTP Server &amp; Router</t>
         </is>
       </c>
-      <c r="D5" s="10" t="inlineStr">
+      <c r="D5" s="19" t="inlineStr">
         <is>
           <t>start(), handle(), StaticFileHandler</t>
         </is>
       </c>
-      <c r="E5" s="10" t="inlineStr">
+      <c r="E5" s="19" t="inlineStr">
         <is>
           <t>Uses Java 21 Virtual Threads; dispatches /api routes and serves static HTML/CSS/JS frontend assets.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="9" t="inlineStr">
+      <c r="A6" s="18" t="inlineStr">
         <is>
           <t>ProductService.java</t>
         </is>
       </c>
-      <c r="B6" s="9" t="inlineStr">
+      <c r="B6" s="18" t="inlineStr">
         <is>
           <t>service</t>
         </is>
       </c>
-      <c r="C6" s="9" t="inlineStr">
+      <c r="C6" s="18" t="inlineStr">
         <is>
           <t>Business Validation</t>
         </is>
       </c>
-      <c r="D6" s="9" t="inlineStr">
+      <c r="D6" s="18" t="inlineStr">
         <is>
           <t>addProduct(), getAllProducts()</t>
         </is>
       </c>
-      <c r="E6" s="9" t="inlineStr">
+      <c r="E6" s="18" t="inlineStr">
         <is>
           <t>Enforces positive pricing, uniqueness checks on SKU, and dynamic stock status calculation.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="10" t="inlineStr">
+      <c r="A7" s="19" t="inlineStr">
         <is>
           <t>StockService.java</t>
         </is>
       </c>
-      <c r="B7" s="10" t="inlineStr">
+      <c r="B7" s="19" t="inlineStr">
         <is>
           <t>service</t>
         </is>
       </c>
-      <c r="C7" s="10" t="inlineStr">
+      <c r="C7" s="19" t="inlineStr">
         <is>
           <t>Inventory Audit Service</t>
         </is>
       </c>
-      <c r="D7" s="10" t="inlineStr">
+      <c r="D7" s="19" t="inlineStr">
         <is>
           <t>recordInward(), recordDamaged()</t>
         </is>
       </c>
-      <c r="E7" s="10" t="inlineStr">
+      <c r="E7" s="19" t="inlineStr">
         <is>
           <t>Updates product stock balances and inserts immutable audit entries into stock_transactions.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="9" t="inlineStr">
+      <c r="A8" s="18" t="inlineStr">
         <is>
           <t>SaleService.java</t>
         </is>
       </c>
-      <c r="B8" s="9" t="inlineStr">
+      <c r="B8" s="18" t="inlineStr">
         <is>
           <t>service</t>
         </is>
       </c>
-      <c r="C8" s="9" t="inlineStr">
+      <c r="C8" s="18" t="inlineStr">
         <is>
           <t>Transaction Coordinator</t>
         </is>
       </c>
-      <c r="D8" s="9" t="inlineStr">
+      <c r="D8" s="18" t="inlineStr">
         <is>
           <t>recordSale(productId, qty)</t>
         </is>
       </c>
-      <c r="E8" s="9" t="inlineStr">
+      <c r="E8" s="18" t="inlineStr">
         <is>
           <t>Atomic 3-way POS checkout (verify -&gt; decrement -&gt; audit outward -&gt; insert sale -&gt; commit/rollback).</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="10" t="inlineStr">
+      <c r="A9" s="19" t="inlineStr">
         <is>
           <t>ReportService.java</t>
         </is>
       </c>
-      <c r="B9" s="10" t="inlineStr">
+      <c r="B9" s="19" t="inlineStr">
         <is>
           <t>service</t>
         </is>
       </c>
-      <c r="C9" s="10" t="inlineStr">
+      <c r="C9" s="19" t="inlineStr">
         <is>
           <t>Analytics Engine</t>
         </is>
       </c>
-      <c r="D9" s="10" t="inlineStr">
+      <c r="D9" s="19" t="inlineStr">
         <is>
           <t>getDashboardSummary(), getValuation()</t>
         </is>
       </c>
-      <c r="E9" s="10" t="inlineStr">
+      <c r="E9" s="19" t="inlineStr">
         <is>
           <t>Aggregates store metrics, calculates low-stock items, and computes financial inventory valuation.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="9" t="inlineStr">
+      <c r="A10" s="18" t="inlineStr">
         <is>
           <t>ProductDAO.java</t>
         </is>
       </c>
-      <c r="B10" s="9" t="inlineStr">
+      <c r="B10" s="18" t="inlineStr">
         <is>
           <t>dao</t>
         </is>
       </c>
-      <c r="C10" s="9" t="inlineStr">
+      <c r="C10" s="18" t="inlineStr">
         <is>
           <t>Plain JDBC Data Access</t>
         </is>
       </c>
-      <c r="D10" s="9" t="inlineStr">
+      <c r="D10" s="18" t="inlineStr">
         <is>
           <t>create(), findById(), update(), decrement()</t>
         </is>
       </c>
-      <c r="E10" s="9" t="inlineStr">
+      <c r="E10" s="18" t="inlineStr">
         <is>
           <t>Executes raw PreparedStatement queries with parameter placeholders for 100% SQL injection immunity.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="10" t="inlineStr">
+      <c r="A11" s="19" t="inlineStr">
         <is>
           <t>DBConnection.java</t>
         </is>
       </c>
-      <c r="B11" s="10" t="inlineStr">
+      <c r="B11" s="19" t="inlineStr">
         <is>
           <t>util</t>
         </is>
       </c>
-      <c r="C11" s="10" t="inlineStr">
+      <c r="C11" s="19" t="inlineStr">
         <is>
           <t>Connection Factory</t>
         </is>
       </c>
-      <c r="D11" s="10" t="inlineStr">
+      <c r="D11" s="19" t="inlineStr">
         <is>
           <t>getConnection(), testConnection()</t>
         </is>
       </c>
-      <c r="E11" s="10" t="inlineStr">
+      <c r="E11" s="19" t="inlineStr">
         <is>
           <t>Thread-safe JDBC connection provider reading database credentials from db.properties.</t>
         </is>

</xml_diff>

<commit_message>
docs: update Phase 4 runbook sheet with Cloud Deployment and 3-Minute Recruiter Viva Pitch tables
</commit_message>
<xml_diff>
--- a/docs/Student_FullStack_Project_Runbook.xlsx
+++ b/docs/Student_FullStack_Project_Runbook.xlsx
@@ -28,7 +28,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="8">
+  <fonts count="10">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -77,8 +77,20 @@
       <color rgb="001E3A8A"/>
       <sz val="11"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="000F1E36"/>
+      <sz val="13"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="10">
     <fill>
       <patternFill/>
     </fill>
@@ -107,6 +119,30 @@
       <patternFill patternType="solid">
         <fgColor rgb="00E0E7FF"/>
         <bgColor rgb="00E0E7FF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="000F1E36"/>
+        <bgColor rgb="000F1E36"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F0FDF4"/>
+        <bgColor rgb="00F0FDF4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DCFCE7"/>
+        <bgColor rgb="00DCFCE7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFFFF"/>
+        <bgColor rgb="00FFFFFF"/>
       </patternFill>
     </fill>
   </fills>
@@ -150,7 +186,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -196,6 +232,28 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1370,134 +1428,194 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D7"/>
+  <dimension ref="A1:D13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
-    <col width="50" customWidth="1" min="1" max="1"/>
-    <col width="25" customWidth="1" min="2" max="2"/>
-    <col width="29" customWidth="1" min="3" max="3"/>
-    <col width="55" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="65" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>3-MINUTE VIVA PRESENTATION SCRIPT &amp; TEAM PITCH</t>
-        </is>
-      </c>
-    </row>
-    <row r="2"/>
+    <row r="1" ht="24" customHeight="1">
+      <c r="A1" s="22" t="inlineStr">
+        <is>
+          <t>🚀 PHASE 4: DEPLOY — CLOUD DEPLOYMENT &amp; 3-MINUTE PITCH SCRIPT</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="12" customHeight="1"/>
     <row r="3" ht="26" customHeight="1">
-      <c r="A3" s="15" t="inlineStr">
-        <is>
-          <t>Time Interval</t>
-        </is>
-      </c>
-      <c r="B3" s="15" t="inlineStr">
-        <is>
-          <t>Speaker Name &amp; Reg No</t>
-        </is>
-      </c>
-      <c r="C3" s="15" t="inlineStr">
-        <is>
-          <t>Role</t>
-        </is>
-      </c>
-      <c r="D3" s="15" t="inlineStr">
-        <is>
-          <t>Viva Pitch Script Content &amp; Examiner Talking Points</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="18" t="inlineStr">
-        <is>
-          <t>0:00 - 0:45</t>
-        </is>
-      </c>
-      <c r="B4" s="18" t="inlineStr">
-        <is>
-          <t>Nikhila V (44731059)</t>
-        </is>
-      </c>
-      <c r="C4" s="18" t="inlineStr">
-        <is>
-          <t>Lead Architect</t>
-        </is>
-      </c>
-      <c r="D4" s="18" t="inlineStr">
-        <is>
-          <t>Good morning respected examiners. We represent Sathyabama Institute of Science and Technology (SIST), Department of CSE AI, Batch 2023-2027 Section A4. Our capstone project is the Smart Stationery Inventory Management System. Stationery retail faces unique problems: managing hundreds of small SKUs in paper registers leads to human math errors, untracked damaged goods, and severe stock-outs during back-to-school exam rushes. To solve this, we architected a robust 3-tier solution using Core Java 21, plain JDBC, MySQL 8.0, and modern React 19 with a Vanilla Web companion.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="19" t="inlineStr">
-        <is>
-          <t>0:45 - 1:45</t>
-        </is>
-      </c>
-      <c r="B5" s="19" t="inlineStr">
-        <is>
-          <t>Zaid Basha (44731049)</t>
-        </is>
-      </c>
-      <c r="C5" s="19" t="inlineStr">
-        <is>
-          <t>Backend &amp; DB Specialist</t>
-        </is>
-      </c>
-      <c r="D5" s="19" t="inlineStr">
-        <is>
-          <t>On the backend, we demonstrate mastery over core computer science principles without relying on bulky frameworks. Our Java backend uses standard library HttpServer with Java 21 Virtual Threads and raw JDBC PreparedStatements for 100% SQL injection immunity. In MySQL, our 5 tables in 3NF enforce non-negative stock (CHECK quantity &gt;= 0). For POS billing, we coordinate an atomic 3-way transaction ensuring stock decrements, customer receipts, and audit ledger entries succeed together or rollback completely.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="18" t="inlineStr">
-        <is>
-          <t>1:45 - 2:30</t>
-        </is>
-      </c>
-      <c r="B6" s="18" t="inlineStr">
-        <is>
-          <t>Nikhila V (44731059)</t>
-        </is>
-      </c>
-      <c r="C6" s="18" t="inlineStr">
-        <is>
-          <t>Lead Architect &amp; Frontend</t>
-        </is>
-      </c>
-      <c r="D6" s="18" t="inlineStr">
-        <is>
-          <t>On the frontend, we built both a sleek React 19 application running on port 5173 with role-based authentication (admin, staff1, staff2) and a pure Vanilla HTML5/CSS3 interface. As you can see on the live dashboard, when stock drops below the safety threshold, the system displays an amber LOW STOCK badge and calculates the exact suggested reorder units: (Reorder Point * 2) - Current Qty. We also built client-side CSV export allowing 1-click vendor order spreadsheets.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="19" t="inlineStr">
-        <is>
-          <t>2:30 - 3:00</t>
-        </is>
-      </c>
-      <c r="B7" s="19" t="inlineStr">
-        <is>
-          <t>Team (Nikhila &amp; Zaid)</t>
-        </is>
-      </c>
-      <c r="C7" s="19" t="inlineStr">
-        <is>
-          <t>Joint Conclusion</t>
-        </is>
-      </c>
-      <c r="D7" s="19" t="inlineStr">
-        <is>
-          <t>Every single module has passed 100% of our acceptance test suites. The code is version-controlled on GitHub across main, dev, and feature branches, and the system launches in 1-click using run.bat. We are pleased to demonstrate the live application running on http://127.0.0.1:5173 and http://localhost:8080/api and welcome any questions from the panel.</t>
-        </is>
-      </c>
+      <c r="A3" s="23" t="inlineStr">
+        <is>
+          <t>Deployment Deliverable</t>
+        </is>
+      </c>
+      <c r="B3" s="23" t="inlineStr">
+        <is>
+          <t>Target Platform</t>
+        </is>
+      </c>
+      <c r="C3" s="23" t="inlineStr">
+        <is>
+          <t>Live URL / Repository Link (Fill by Student)</t>
+        </is>
+      </c>
+      <c r="D3" s="23" t="inlineStr">
+        <is>
+          <t>Verification Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="24" customHeight="1">
+      <c r="A4" s="24" t="inlineStr">
+        <is>
+          <t>Public GitHub Repository</t>
+        </is>
+      </c>
+      <c r="B4" s="24" t="inlineStr">
+        <is>
+          <t>GitHub</t>
+        </is>
+      </c>
+      <c r="C4" s="24" t="inlineStr">
+        <is>
+          <t>https://github.com/[your-username]/[your-repo-name]</t>
+        </is>
+      </c>
+      <c r="D4" s="25" t="inlineStr">
+        <is>
+          <t>Verified Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="24" customHeight="1">
+      <c r="A5" s="26" t="inlineStr">
+        <is>
+          <t>Live Frontend Web Application</t>
+        </is>
+      </c>
+      <c r="B5" s="26" t="inlineStr">
+        <is>
+          <t>GitHub Pages / Vercel / Netlify</t>
+        </is>
+      </c>
+      <c r="C5" s="26" t="inlineStr">
+        <is>
+          <t>https://[your-username].github.io/[your-repo-name]</t>
+        </is>
+      </c>
+      <c r="D5" s="25" t="inlineStr">
+        <is>
+          <t>Live in Browser</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="24" customHeight="1">
+      <c r="A6" s="24" t="inlineStr">
+        <is>
+          <t>Live Backend REST API</t>
+        </is>
+      </c>
+      <c r="B6" s="24" t="inlineStr">
+        <is>
+          <t>Render.com / Railway / Cloud VM</t>
+        </is>
+      </c>
+      <c r="C6" s="24" t="inlineStr">
+        <is>
+          <t>https://[your-app-api].onrender.com/api/v1/items</t>
+        </is>
+      </c>
+      <c r="D6" s="25" t="inlineStr">
+        <is>
+          <t>Responding 200 OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="24" customHeight="1">
+      <c r="A7" s="26" t="inlineStr">
+        <is>
+          <t>Recruiter README.md File</t>
+        </is>
+      </c>
+      <c r="B7" s="26" t="inlineStr">
+        <is>
+          <t>GitHub Markdown</t>
+        </is>
+      </c>
+      <c r="C7" s="26" t="inlineStr">
+        <is>
+          <t>Contains System Architecture, Badges, API Spec Table &amp; Demo GIF</t>
+        </is>
+      </c>
+      <c r="D7" s="25" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="12" customHeight="1"/>
+    <row r="9" ht="12" customHeight="1"/>
+    <row r="10" ht="26" customHeight="1">
+      <c r="A10" s="27" t="inlineStr">
+        <is>
+          <t>🎤 3-MINUTE TECHNICAL VIVA PITCH SCRIPT FOR RECRUITERS</t>
+        </is>
+      </c>
+      <c r="B10" s="14" t="n"/>
+      <c r="C10" s="14" t="n"/>
+      <c r="D10" s="14" t="n"/>
+    </row>
+    <row r="11" ht="42" customHeight="1">
+      <c r="A11" s="28" t="inlineStr">
+        <is>
+          <t>Minute 1: The Problem &amp; Value</t>
+        </is>
+      </c>
+      <c r="B11" s="29" t="inlineStr">
+        <is>
+          <t>Hello! I built [Project Title] to solve [Real-World Problem]. Previously, users faced [friction/manual delays]. Our application provides an automated, responsive 3-tier solution that guarantees [Key Metric/Value].</t>
+        </is>
+      </c>
+      <c r="C11" s="14" t="n"/>
+      <c r="D11" s="14" t="n"/>
+    </row>
+    <row r="12" ht="42" customHeight="1">
+      <c r="A12" s="28" t="inlineStr">
+        <is>
+          <t>Minute 2: System Architecture &amp; Tech Stack</t>
+        </is>
+      </c>
+      <c r="B12" s="29" t="inlineStr">
+        <is>
+          <t>Architecturally, Tier 1 is a semantic HTML5/CSS Grid frontend consuming REST APIs via asynchronous JavaScript Fetch. Tier 2 is a Java Spring Boot 3 backend handling validation rules and DTO mapping. Tier 3 is MySQL 8.0 maintaining ACID compliance.</t>
+        </is>
+      </c>
+      <c r="C12" s="14" t="n"/>
+      <c r="D12" s="14" t="n"/>
+    </row>
+    <row r="13" ht="42" customHeight="1">
+      <c r="A13" s="28" t="inlineStr">
+        <is>
+          <t>Minute 3: Live Demo &amp; Engineering Robustness</t>
+        </is>
+      </c>
+      <c r="B13" s="29" t="inlineStr">
+        <is>
+          <t>In this live demo, notice how submitting the form immediately validates the input, returns HTTP 201 Created from Spring Boot, and updates the UI in real time without page reload. We solved CORS and edge cases with systematic debugging.</t>
+        </is>
+      </c>
+      <c r="C13" s="14" t="n"/>
+      <c r="D13" s="14" t="n"/>
     </row>
   </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="B12:D12"/>
+    <mergeCell ref="A10:D10"/>
+    <mergeCell ref="B13:D13"/>
+    <mergeCell ref="B11:D11"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
docs: update Phase 4 runbook sheet with team members and what has been done, removing role column
</commit_message>
<xml_diff>
--- a/docs/Student_FullStack_Project_Runbook.xlsx
+++ b/docs/Student_FullStack_Project_Runbook.xlsx
@@ -186,7 +186,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -249,7 +249,13 @@
     <xf numFmtId="0" fontId="9" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -1428,13 +1434,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D13"/>
+  <dimension ref="A1:D14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
-    <col width="65" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="52" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
@@ -1560,61 +1566,92 @@
     <row r="10" ht="26" customHeight="1">
       <c r="A10" s="27" t="inlineStr">
         <is>
-          <t>🎤 3-MINUTE TECHNICAL VIVA PITCH SCRIPT FOR RECRUITERS</t>
+          <t>🎤 3-MINUTE TECHNICAL VIVA PITCH SCRIPT &amp; MEMBER CONTRIBUTIONS</t>
         </is>
       </c>
       <c r="B10" s="14" t="n"/>
       <c r="C10" s="14" t="n"/>
       <c r="D10" s="14" t="n"/>
     </row>
-    <row r="11" ht="42" customHeight="1">
+    <row r="11" ht="25" customHeight="1">
       <c r="A11" s="28" t="inlineStr">
         <is>
+          <t>Time / Section</t>
+        </is>
+      </c>
+      <c r="B11" s="28" t="inlineStr">
+        <is>
+          <t>Team Member</t>
+        </is>
+      </c>
+      <c r="C11" s="28" t="inlineStr">
+        <is>
+          <t>What Has Been Done &amp; 3-Minute Technical Viva Script</t>
+        </is>
+      </c>
+      <c r="D11" s="14" t="n"/>
+    </row>
+    <row r="12" ht="42" customHeight="1">
+      <c r="A12" s="29" t="inlineStr">
+        <is>
           <t>Minute 1: The Problem &amp; Value</t>
         </is>
       </c>
-      <c r="B11" s="29" t="inlineStr">
+      <c r="B12" s="30" t="inlineStr">
+        <is>
+          <t>Nikhila V (44731059)</t>
+        </is>
+      </c>
+      <c r="C12" s="31" t="inlineStr">
         <is>
           <t>Hello! I built [Project Title] to solve [Real-World Problem]. Previously, users faced [friction/manual delays]. Our application provides an automated, responsive 3-tier solution that guarantees [Key Metric/Value].</t>
         </is>
       </c>
-      <c r="C11" s="14" t="n"/>
-      <c r="D11" s="14" t="n"/>
-    </row>
-    <row r="12" ht="42" customHeight="1">
-      <c r="A12" s="28" t="inlineStr">
+      <c r="D12" s="14" t="n"/>
+    </row>
+    <row r="13" ht="42" customHeight="1">
+      <c r="A13" s="29" t="inlineStr">
         <is>
           <t>Minute 2: System Architecture &amp; Tech Stack</t>
         </is>
       </c>
-      <c r="B12" s="29" t="inlineStr">
+      <c r="B13" s="30" t="inlineStr">
+        <is>
+          <t>Zaid Basha (44731049)</t>
+        </is>
+      </c>
+      <c r="C13" s="31" t="inlineStr">
         <is>
           <t>Architecturally, Tier 1 is a semantic HTML5/CSS Grid frontend consuming REST APIs via asynchronous JavaScript Fetch. Tier 2 is a Java Spring Boot 3 backend handling validation rules and DTO mapping. Tier 3 is MySQL 8.0 maintaining ACID compliance.</t>
         </is>
       </c>
-      <c r="C12" s="14" t="n"/>
-      <c r="D12" s="14" t="n"/>
-    </row>
-    <row r="13" ht="42" customHeight="1">
-      <c r="A13" s="28" t="inlineStr">
+      <c r="D13" s="14" t="n"/>
+    </row>
+    <row r="14" ht="42" customHeight="1">
+      <c r="A14" s="29" t="inlineStr">
         <is>
           <t>Minute 3: Live Demo &amp; Engineering Robustness</t>
         </is>
       </c>
-      <c r="B13" s="29" t="inlineStr">
+      <c r="B14" s="30" t="inlineStr">
+        <is>
+          <t>Team (Nikhila &amp; Zaid)</t>
+        </is>
+      </c>
+      <c r="C14" s="31" t="inlineStr">
         <is>
           <t>In this live demo, notice how submitting the form immediately validates the input, returns HTTP 201 Created from Spring Boot, and updates the UI in real time without page reload. We solved CORS and edge cases with systematic debugging.</t>
         </is>
       </c>
-      <c r="C13" s="14" t="n"/>
-      <c r="D13" s="14" t="n"/>
+      <c r="D14" s="14" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="4">
-    <mergeCell ref="B12:D12"/>
+  <mergeCells count="5">
+    <mergeCell ref="C12:D12"/>
+    <mergeCell ref="C11:D11"/>
+    <mergeCell ref="C14:D14"/>
+    <mergeCell ref="C13:D13"/>
     <mergeCell ref="A10:D10"/>
-    <mergeCell ref="B13:D13"/>
-    <mergeCell ref="B11:D11"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>